<commit_message>
Implement User Management UI and access control
</commit_message>
<xml_diff>
--- a/PMO_Master.xlsx
+++ b/PMO_Master.xlsx
@@ -525,7 +525,7 @@
         <v>Overall Progress</v>
       </c>
     </row>
-    <row r="2" xml:space="preserve">
+    <row r="2">
       <c r="A2" t="str">
         <v/>
       </c>
@@ -577,9 +577,8 @@
       <c r="Q2" t="str">
         <v>N</v>
       </c>
-      <c r="R2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Please get this work done
-</v>
+      <c r="R2" t="str">
+        <v>Please get this work done</v>
       </c>
       <c r="S2" t="str">
         <v/>
@@ -614,9 +613,8 @@
       <c r="AC2" t="str">
         <v/>
       </c>
-      <c r="AD2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Please get this work done
-</v>
+      <c r="AD2" t="str">
+        <v>Please get this work done</v>
       </c>
     </row>
     <row r="3">
@@ -675,10 +673,10 @@
         <v>20% complete</v>
       </c>
       <c r="S3" t="str">
-        <v>2025-03-01</v>
+        <v>2025-03-10</v>
       </c>
       <c r="T3" t="str">
-        <v>2025-04-30</v>
+        <v>2025-04-25</v>
       </c>
       <c r="U3" t="str">
         <v>2025-05-01</v>

</xml_diff>

<commit_message>
Implement 4-date system, Gantt dual-tracks, and Flagship theme merging
</commit_message>
<xml_diff>
--- a/PMO_Master.xlsx
+++ b/PMO_Master.xlsx
@@ -1011,7 +1011,7 @@
         <v>2025-12-31</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>2026-01-12</v>
       </c>
       <c r="J7">
         <v>160</v>
@@ -1065,10 +1065,10 @@
         <v>2025-12-31</v>
       </c>
       <c r="AA7" t="str">
-        <v/>
+        <v>2026-02-12</v>
       </c>
       <c r="AB7" t="str">
-        <v/>
+        <v>2026-04-12</v>
       </c>
       <c r="AC7" t="str">
         <v/>

</xml_diff>

<commit_message>
Update Excel Sync to export/import all 4 dates for phases
</commit_message>
<xml_diff>
--- a/PMO_Master.xlsx
+++ b/PMO_Master.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD13"/>
+  <dimension ref="A1:AN12"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -419,18 +419,8 @@
     <col min="16" max="16" width="16.83203125" customWidth="1"/>
     <col min="17" max="17" width="19.83203125" customWidth="1"/>
     <col min="18" max="18" width="16.83203125" customWidth="1"/>
-    <col min="19" max="19" width="17.83203125" customWidth="1"/>
-    <col min="20" max="20" width="16.83203125" customWidth="1"/>
-    <col min="21" max="21" width="17.83203125" customWidth="1"/>
-    <col min="22" max="22" width="16.83203125" customWidth="1"/>
-    <col min="23" max="23" width="17.83203125" customWidth="1"/>
-    <col min="24" max="24" width="16.83203125" customWidth="1"/>
-    <col min="25" max="25" width="17.83203125" customWidth="1"/>
-    <col min="26" max="26" width="16.83203125" customWidth="1"/>
-    <col min="27" max="27" width="17.83203125" customWidth="1"/>
-    <col min="28" max="28" width="16.83203125" customWidth="1"/>
-    <col min="29" max="29" width="22.83203125" customWidth="1"/>
-    <col min="30" max="30" width="18.83203125" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="20" max="20" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -489,84 +479,54 @@
         <v>Remarks</v>
       </c>
       <c r="S1" t="str">
-        <v>IL1 Phase Start</v>
+        <v>Assigned To Staff ID</v>
       </c>
       <c r="T1" t="str">
-        <v>IL1 Phase End</v>
-      </c>
-      <c r="U1" t="str">
-        <v>IL2 Phase Start</v>
-      </c>
-      <c r="V1" t="str">
-        <v>IL2 Phase End</v>
-      </c>
-      <c r="W1" t="str">
-        <v>IL3 Phase Start</v>
-      </c>
-      <c r="X1" t="str">
-        <v>IL3 Phase End</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>IL4 Phase Start</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>IL4 Phase End</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>IL5 Phase Start</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>IL5 Phase End</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>Assigned To Staff ID</v>
-      </c>
-      <c r="AD1" t="str">
         <v>Overall Progress</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>MSL-002</v>
       </c>
       <c r="B2" t="str">
-        <v>kartavya</v>
+        <v>SAP HR Module Integration</v>
       </c>
       <c r="C2" t="str">
-        <v>Customer Experience</v>
+        <v>Operational Excellence</v>
       </c>
       <c r="D2" t="str">
-        <v>Finance</v>
+        <v>HR</v>
       </c>
       <c r="E2" t="str">
-        <v>IL3</v>
+        <v>IL2</v>
       </c>
       <c r="F2" t="str">
-        <v>Customer Facing</v>
+        <v>Integration</v>
       </c>
       <c r="G2" t="str">
         <v>2025-26</v>
       </c>
       <c r="H2" t="str">
-        <v>2029-08-23</v>
+        <v>2026-03-31</v>
       </c>
       <c r="I2" t="str">
-        <v>2030-08-23</v>
+        <v/>
       </c>
       <c r="J2">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="K2">
-        <v>123</v>
-      </c>
-      <c r="L2">
-        <v>123</v>
+        <v>1200000</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
       </c>
       <c r="M2">
-        <v>123</v>
+        <v>12</v>
       </c>
       <c r="N2" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="O2" t="str">
         <v>N</v>
@@ -575,10 +535,10 @@
         <v>Y</v>
       </c>
       <c r="Q2" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="R2" t="str">
-        <v>Please get this work done</v>
+        <v>20% complete</v>
       </c>
       <c r="S2" t="str">
         <v/>
@@ -614,51 +574,81 @@
         <v/>
       </c>
       <c r="AD2" t="str">
-        <v>Please get this work done</v>
+        <v/>
+      </c>
+      <c r="AE2" t="str">
+        <v/>
+      </c>
+      <c r="AF2" t="str">
+        <v/>
+      </c>
+      <c r="AG2" t="str">
+        <v/>
+      </c>
+      <c r="AH2" t="str">
+        <v/>
+      </c>
+      <c r="AI2" t="str">
+        <v/>
+      </c>
+      <c r="AJ2" t="str">
+        <v/>
+      </c>
+      <c r="AK2" t="str">
+        <v/>
+      </c>
+      <c r="AL2" t="str">
+        <v/>
+      </c>
+      <c r="AM2" t="str">
+        <v/>
+      </c>
+      <c r="AN2" t="str">
+        <v>20% complete</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>MSL-002</v>
+        <v>MSL-003</v>
       </c>
       <c r="B3" t="str">
-        <v>SAP HR Module Integration</v>
+        <v>Customer Complaint Analytics</v>
       </c>
       <c r="C3" t="str">
-        <v>Operational Excellence</v>
+        <v>Customer Experience</v>
       </c>
       <c r="D3" t="str">
-        <v>HR</v>
+        <v>Customer Service</v>
       </c>
       <c r="E3" t="str">
-        <v>IL2</v>
+        <v>IL4</v>
       </c>
       <c r="F3" t="str">
-        <v>Integration</v>
+        <v>Analytics</v>
       </c>
       <c r="G3" t="str">
-        <v>2025-26</v>
+        <v>2024-25</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-03-31</v>
+        <v>2025-06-30</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>2025-07-15</v>
       </c>
       <c r="J3">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="K3">
-        <v>1200000</v>
-      </c>
-      <c r="L3" t="str">
-        <v/>
+        <v>340000</v>
+      </c>
+      <c r="L3">
+        <v>55</v>
       </c>
       <c r="M3">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="N3" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="O3" t="str">
         <v>N</v>
@@ -670,16 +660,16 @@
         <v>Y</v>
       </c>
       <c r="R3" t="str">
-        <v>20% complete</v>
+        <v>95% — live this week</v>
       </c>
       <c r="S3" t="str">
-        <v>2025-03-10</v>
+        <v/>
       </c>
       <c r="T3" t="str">
-        <v>2025-04-25</v>
+        <v/>
       </c>
       <c r="U3" t="str">
-        <v>2025-05-01</v>
+        <v/>
       </c>
       <c r="V3" t="str">
         <v/>
@@ -706,99 +696,159 @@
         <v/>
       </c>
       <c r="AD3" t="str">
-        <v>20% complete</v>
+        <v/>
+      </c>
+      <c r="AE3" t="str">
+        <v/>
+      </c>
+      <c r="AF3" t="str">
+        <v/>
+      </c>
+      <c r="AG3" t="str">
+        <v/>
+      </c>
+      <c r="AH3" t="str">
+        <v/>
+      </c>
+      <c r="AI3" t="str">
+        <v/>
+      </c>
+      <c r="AJ3" t="str">
+        <v/>
+      </c>
+      <c r="AK3" t="str">
+        <v/>
+      </c>
+      <c r="AL3" t="str">
+        <v/>
+      </c>
+      <c r="AM3" t="str">
+        <v/>
+      </c>
+      <c r="AN3" t="str">
+        <v>95% — live this week</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MSL-003</v>
+        <v>MSL-005</v>
       </c>
       <c r="B4" t="str">
-        <v>Customer Complaint Analytics</v>
+        <v>Mobile Approval Workflow App</v>
       </c>
       <c r="C4" t="str">
-        <v>Customer Experience</v>
+        <v>Digital Transformation</v>
       </c>
       <c r="D4" t="str">
-        <v>Customer Service</v>
+        <v>IT</v>
       </c>
       <c r="E4" t="str">
-        <v>IL4</v>
+        <v>IL1</v>
       </c>
       <c r="F4" t="str">
-        <v>Analytics</v>
+        <v>Innovation</v>
       </c>
       <c r="G4" t="str">
-        <v>2024-25</v>
+        <v>2026-27</v>
       </c>
       <c r="H4" t="str">
-        <v>2025-06-30</v>
+        <v>2026-09-30</v>
       </c>
       <c r="I4" t="str">
-        <v>2025-07-15</v>
+        <v/>
       </c>
       <c r="J4">
-        <v>80</v>
-      </c>
-      <c r="K4">
-        <v>340000</v>
-      </c>
-      <c r="L4">
-        <v>55</v>
+        <v>60</v>
+      </c>
+      <c r="K4" t="str">
+        <v/>
+      </c>
+      <c r="L4" t="str">
+        <v/>
       </c>
       <c r="M4">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="N4" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="O4" t="str">
         <v>N</v>
       </c>
       <c r="P4" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="Q4" t="str">
         <v>N</v>
       </c>
       <c r="R4" t="str">
-        <v>95% — live this week</v>
+        <v>10% — ideation</v>
       </c>
       <c r="S4" t="str">
-        <v>2024-10-01</v>
+        <v/>
       </c>
       <c r="T4" t="str">
-        <v>2024-11-30</v>
+        <v/>
       </c>
       <c r="U4" t="str">
-        <v>2024-12-01</v>
+        <v/>
       </c>
       <c r="V4" t="str">
-        <v>2025-01-31</v>
+        <v/>
       </c>
       <c r="W4" t="str">
-        <v>2025-02-01</v>
+        <v/>
       </c>
       <c r="X4" t="str">
-        <v>2025-04-30</v>
+        <v/>
       </c>
       <c r="Y4" t="str">
-        <v>2025-05-01</v>
+        <v/>
       </c>
       <c r="Z4" t="str">
-        <v>2025-06-30</v>
+        <v/>
       </c>
       <c r="AA4" t="str">
-        <v>2026-06-01</v>
+        <v/>
       </c>
       <c r="AB4" t="str">
-        <v>2026-07-15</v>
+        <v/>
       </c>
       <c r="AC4" t="str">
         <v/>
       </c>
       <c r="AD4" t="str">
-        <v>95% — live this week</v>
+        <v/>
+      </c>
+      <c r="AE4" t="str">
+        <v/>
+      </c>
+      <c r="AF4" t="str">
+        <v/>
+      </c>
+      <c r="AG4" t="str">
+        <v/>
+      </c>
+      <c r="AH4" t="str">
+        <v/>
+      </c>
+      <c r="AI4" t="str">
+        <v/>
+      </c>
+      <c r="AJ4" t="str">
+        <v/>
+      </c>
+      <c r="AK4" t="str">
+        <v/>
+      </c>
+      <c r="AL4" t="str">
+        <v/>
+      </c>
+      <c r="AM4" t="str">
+        <v/>
+      </c>
+      <c r="AN4" t="str">
+        <v>10% — ideation</v>
       </c>
     </row>
     <row r="5">
@@ -857,99 +907,129 @@
         <v>100% — Live &amp; stable</v>
       </c>
       <c r="S5" t="str">
-        <v>2024-07-01</v>
+        <v>2024-02-15</v>
       </c>
       <c r="T5" t="str">
-        <v>2024-08-15</v>
+        <v/>
       </c>
       <c r="U5" t="str">
-        <v>2024-08-01</v>
+        <v>2024-06-13</v>
       </c>
       <c r="V5" t="str">
-        <v>2024-10-31</v>
+        <v/>
       </c>
       <c r="W5" t="str">
-        <v>2024-11-01</v>
+        <v/>
       </c>
       <c r="X5" t="str">
-        <v>2025-01-31</v>
+        <v/>
       </c>
       <c r="Y5" t="str">
-        <v>2025-02-01</v>
+        <v/>
       </c>
       <c r="Z5" t="str">
-        <v>2025-03-15</v>
+        <v/>
       </c>
       <c r="AA5" t="str">
-        <v>2025-03-16</v>
+        <v/>
       </c>
       <c r="AB5" t="str">
-        <v>2025-03-28</v>
+        <v/>
       </c>
       <c r="AC5" t="str">
         <v/>
       </c>
       <c r="AD5" t="str">
+        <v/>
+      </c>
+      <c r="AE5" t="str">
+        <v/>
+      </c>
+      <c r="AF5" t="str">
+        <v/>
+      </c>
+      <c r="AG5" t="str">
+        <v/>
+      </c>
+      <c r="AH5" t="str">
+        <v/>
+      </c>
+      <c r="AI5" t="str">
+        <v/>
+      </c>
+      <c r="AJ5" t="str">
+        <v/>
+      </c>
+      <c r="AK5" t="str">
+        <v/>
+      </c>
+      <c r="AL5" t="str">
+        <v/>
+      </c>
+      <c r="AM5" t="str">
+        <v/>
+      </c>
+      <c r="AN5" t="str">
         <v>100% — Live &amp; stable</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MSL-005</v>
+        <v>MSL-001</v>
       </c>
       <c r="B6" t="str">
-        <v>Mobile Approval Workflow App</v>
+        <v>Vendor Portal Digitization</v>
       </c>
       <c r="C6" t="str">
         <v>Digital Transformation</v>
       </c>
       <c r="D6" t="str">
-        <v>IT</v>
+        <v>Finance</v>
       </c>
       <c r="E6" t="str">
         <v>IL3</v>
       </c>
       <c r="F6" t="str">
-        <v>Innovation</v>
+        <v>Process Automation</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-27</v>
+        <v>2025-26</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-09-30</v>
+        <v>2025-12-31</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>2026-01-12</v>
       </c>
       <c r="J6">
-        <v>60</v>
-      </c>
-      <c r="K6" t="str">
-        <v/>
-      </c>
-      <c r="L6" t="str">
-        <v/>
+        <v>160</v>
+      </c>
+      <c r="K6">
+        <v>850000</v>
+      </c>
+      <c r="L6">
+        <v>38</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N6" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="O6" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="P6" t="str">
         <v>N</v>
       </c>
       <c r="Q6" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="R6" t="str">
-        <v>10% — ideation</v>
+        <v>65% complete</v>
       </c>
       <c r="S6" t="str">
-        <v>2026-04-01</v>
+        <v/>
       </c>
       <c r="T6" t="str">
         <v/>
@@ -982,143 +1062,203 @@
         <v/>
       </c>
       <c r="AD6" t="str">
-        <v>10% — ideation</v>
+        <v/>
+      </c>
+      <c r="AE6" t="str">
+        <v/>
+      </c>
+      <c r="AF6" t="str">
+        <v/>
+      </c>
+      <c r="AG6" t="str">
+        <v/>
+      </c>
+      <c r="AH6" t="str">
+        <v/>
+      </c>
+      <c r="AI6" t="str">
+        <v/>
+      </c>
+      <c r="AJ6" t="str">
+        <v/>
+      </c>
+      <c r="AK6" t="str">
+        <v/>
+      </c>
+      <c r="AL6" t="str">
+        <v/>
+      </c>
+      <c r="AM6" t="str">
+        <v/>
+      </c>
+      <c r="AN6" t="str">
+        <v>65% complete</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MSL-001</v>
+        <v>MSL-002</v>
       </c>
       <c r="B7" t="str">
-        <v>Vendor Portal Digitization</v>
+        <v>SAP HR Module Integration</v>
       </c>
       <c r="C7" t="str">
-        <v>Digital Transformation</v>
+        <v>Operational Excellence</v>
       </c>
       <c r="D7" t="str">
-        <v>Finance</v>
+        <v>HR</v>
       </c>
       <c r="E7" t="str">
-        <v>IL3</v>
+        <v>IL2</v>
       </c>
       <c r="F7" t="str">
-        <v>Process Automation</v>
+        <v>Integration</v>
       </c>
       <c r="G7" t="str">
         <v>2025-26</v>
       </c>
       <c r="H7" t="str">
-        <v>2025-12-31</v>
+        <v>2026-03-31</v>
       </c>
       <c r="I7" t="str">
-        <v>2026-01-12</v>
+        <v/>
       </c>
       <c r="J7">
-        <v>160</v>
+        <v>120</v>
       </c>
       <c r="K7">
-        <v>850000</v>
-      </c>
-      <c r="L7">
-        <v>38</v>
+        <v>1200000</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
       </c>
       <c r="M7">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="N7" t="str">
+        <v>N</v>
+      </c>
+      <c r="O7" t="str">
+        <v>N</v>
+      </c>
+      <c r="P7" t="str">
         <v>Y</v>
-      </c>
-      <c r="O7" t="str">
-        <v>Y</v>
-      </c>
-      <c r="P7" t="str">
-        <v>N</v>
       </c>
       <c r="Q7" t="str">
         <v>Y</v>
       </c>
       <c r="R7" t="str">
-        <v>65% complete</v>
+        <v>20% complete</v>
       </c>
       <c r="S7" t="str">
-        <v>2025-04-01</v>
+        <v/>
       </c>
       <c r="T7" t="str">
-        <v>2025-05-15</v>
+        <v/>
       </c>
       <c r="U7" t="str">
-        <v>2025-05-01</v>
+        <v/>
       </c>
       <c r="V7" t="str">
-        <v>2025-07-31</v>
+        <v/>
       </c>
       <c r="W7" t="str">
-        <v>2025-08-01</v>
+        <v/>
       </c>
       <c r="X7" t="str">
-        <v>2025-11-30</v>
+        <v/>
       </c>
       <c r="Y7" t="str">
-        <v>2025-12-01</v>
+        <v/>
       </c>
       <c r="Z7" t="str">
-        <v>2025-12-31</v>
+        <v/>
       </c>
       <c r="AA7" t="str">
-        <v>2026-02-12</v>
+        <v/>
       </c>
       <c r="AB7" t="str">
-        <v>2026-04-12</v>
+        <v/>
       </c>
       <c r="AC7" t="str">
         <v/>
       </c>
       <c r="AD7" t="str">
-        <v>65% complete</v>
+        <v/>
+      </c>
+      <c r="AE7" t="str">
+        <v/>
+      </c>
+      <c r="AF7" t="str">
+        <v/>
+      </c>
+      <c r="AG7" t="str">
+        <v/>
+      </c>
+      <c r="AH7" t="str">
+        <v/>
+      </c>
+      <c r="AI7" t="str">
+        <v/>
+      </c>
+      <c r="AJ7" t="str">
+        <v/>
+      </c>
+      <c r="AK7" t="str">
+        <v/>
+      </c>
+      <c r="AL7" t="str">
+        <v/>
+      </c>
+      <c r="AM7" t="str">
+        <v/>
+      </c>
+      <c r="AN7" t="str">
+        <v>20% complete</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MSL-002</v>
+        <v>MSL-003</v>
       </c>
       <c r="B8" t="str">
-        <v>SAP HR Module Integration</v>
+        <v>Customer Complaint Analytics</v>
       </c>
       <c r="C8" t="str">
-        <v>Operational Excellence</v>
+        <v>Customer Experience</v>
       </c>
       <c r="D8" t="str">
-        <v>HR</v>
+        <v>Customer Service</v>
       </c>
       <c r="E8" t="str">
-        <v>IL2</v>
+        <v>IL4</v>
       </c>
       <c r="F8" t="str">
-        <v>Integration</v>
+        <v>Analytics</v>
       </c>
       <c r="G8" t="str">
-        <v>2025-26</v>
+        <v>2024-25</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-03-31</v>
+        <v>2025-06-30</v>
       </c>
       <c r="I8" t="str">
-        <v/>
+        <v>2025-07-15</v>
       </c>
       <c r="J8">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="K8">
-        <v>1200000</v>
-      </c>
-      <c r="L8" t="str">
-        <v/>
+        <v>340000</v>
+      </c>
+      <c r="L8">
+        <v>55</v>
       </c>
       <c r="M8">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="N8" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="O8" t="str">
         <v>N</v>
@@ -1130,16 +1270,16 @@
         <v>Y</v>
       </c>
       <c r="R8" t="str">
-        <v>20% complete</v>
+        <v>95% — live this week</v>
       </c>
       <c r="S8" t="str">
-        <v>2025-03-01</v>
+        <v/>
       </c>
       <c r="T8" t="str">
-        <v>2025-04-30</v>
+        <v/>
       </c>
       <c r="U8" t="str">
-        <v>2025-05-01</v>
+        <v/>
       </c>
       <c r="V8" t="str">
         <v/>
@@ -1166,54 +1306,84 @@
         <v/>
       </c>
       <c r="AD8" t="str">
-        <v>20% complete</v>
+        <v/>
+      </c>
+      <c r="AE8" t="str">
+        <v/>
+      </c>
+      <c r="AF8" t="str">
+        <v/>
+      </c>
+      <c r="AG8" t="str">
+        <v/>
+      </c>
+      <c r="AH8" t="str">
+        <v/>
+      </c>
+      <c r="AI8" t="str">
+        <v/>
+      </c>
+      <c r="AJ8" t="str">
+        <v/>
+      </c>
+      <c r="AK8" t="str">
+        <v/>
+      </c>
+      <c r="AL8" t="str">
+        <v/>
+      </c>
+      <c r="AM8" t="str">
+        <v/>
+      </c>
+      <c r="AN8" t="str">
+        <v>95% — live this week</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>MSL-003</v>
+        <v>MSL-004</v>
       </c>
       <c r="B9" t="str">
-        <v>Customer Complaint Analytics</v>
+        <v>Supply Chain Visibility Dashboard</v>
       </c>
       <c r="C9" t="str">
-        <v>Customer Experience</v>
+        <v>Data &amp; Analytics</v>
       </c>
       <c r="D9" t="str">
-        <v>Customer Service</v>
+        <v>Supply Chain</v>
       </c>
       <c r="E9" t="str">
-        <v>IL4</v>
+        <v>Live</v>
       </c>
       <c r="F9" t="str">
-        <v>Analytics</v>
+        <v>Reporting</v>
       </c>
       <c r="G9" t="str">
         <v>2024-25</v>
       </c>
       <c r="H9" t="str">
-        <v>2025-06-30</v>
+        <v>2025-03-31</v>
       </c>
       <c r="I9" t="str">
-        <v>2025-07-15</v>
+        <v>2025-03-28</v>
       </c>
       <c r="J9">
-        <v>80</v>
+        <v>200</v>
       </c>
       <c r="K9">
-        <v>340000</v>
+        <v>675000</v>
       </c>
       <c r="L9">
-        <v>55</v>
+        <v>72</v>
       </c>
       <c r="M9">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="N9" t="str">
         <v>Y</v>
       </c>
       <c r="O9" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="P9" t="str">
         <v>Y</v>
@@ -1222,179 +1392,239 @@
         <v>N</v>
       </c>
       <c r="R9" t="str">
-        <v>95% — live this week</v>
+        <v>100% — Live &amp; stable</v>
       </c>
       <c r="S9" t="str">
-        <v>2024-10-01</v>
+        <v/>
       </c>
       <c r="T9" t="str">
-        <v>2024-11-30</v>
+        <v/>
       </c>
       <c r="U9" t="str">
-        <v>2024-12-01</v>
+        <v/>
       </c>
       <c r="V9" t="str">
-        <v>2025-01-31</v>
+        <v/>
       </c>
       <c r="W9" t="str">
-        <v>2025-02-01</v>
+        <v/>
       </c>
       <c r="X9" t="str">
-        <v>2025-04-30</v>
+        <v/>
       </c>
       <c r="Y9" t="str">
-        <v>2025-05-01</v>
+        <v/>
       </c>
       <c r="Z9" t="str">
-        <v>2025-06-30</v>
+        <v/>
       </c>
       <c r="AA9" t="str">
-        <v>2025-07-01</v>
+        <v/>
       </c>
       <c r="AB9" t="str">
-        <v>2025-07-15</v>
+        <v/>
       </c>
       <c r="AC9" t="str">
         <v/>
       </c>
       <c r="AD9" t="str">
-        <v>95% — live this week</v>
+        <v/>
+      </c>
+      <c r="AE9" t="str">
+        <v/>
+      </c>
+      <c r="AF9" t="str">
+        <v/>
+      </c>
+      <c r="AG9" t="str">
+        <v/>
+      </c>
+      <c r="AH9" t="str">
+        <v/>
+      </c>
+      <c r="AI9" t="str">
+        <v/>
+      </c>
+      <c r="AJ9" t="str">
+        <v/>
+      </c>
+      <c r="AK9" t="str">
+        <v/>
+      </c>
+      <c r="AL9" t="str">
+        <v/>
+      </c>
+      <c r="AM9" t="str">
+        <v/>
+      </c>
+      <c r="AN9" t="str">
+        <v>100% — Live &amp; stable</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>MSL-004</v>
+        <v>MSL-005</v>
       </c>
       <c r="B10" t="str">
-        <v>Supply Chain Visibility Dashboard</v>
+        <v>Mobile Approval Workflow App</v>
       </c>
       <c r="C10" t="str">
-        <v>Data &amp; Analytics</v>
+        <v>Digital Transformation</v>
       </c>
       <c r="D10" t="str">
-        <v>Supply Chain</v>
+        <v>IT</v>
       </c>
       <c r="E10" t="str">
-        <v>Live</v>
+        <v>IL1</v>
       </c>
       <c r="F10" t="str">
-        <v>Reporting</v>
+        <v>Innovation</v>
       </c>
       <c r="G10" t="str">
-        <v>2024-25</v>
+        <v>2026-27</v>
       </c>
       <c r="H10" t="str">
-        <v>2025-03-31</v>
+        <v>2026-09-30</v>
       </c>
       <c r="I10" t="str">
-        <v>2025-03-28</v>
+        <v/>
       </c>
       <c r="J10">
-        <v>200</v>
-      </c>
-      <c r="K10">
-        <v>675000</v>
-      </c>
-      <c r="L10">
-        <v>72</v>
+        <v>60</v>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
+        <v/>
       </c>
       <c r="M10">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="N10" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="O10" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="P10" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="Q10" t="str">
         <v>N</v>
       </c>
       <c r="R10" t="str">
-        <v>100% — Live &amp; stable</v>
+        <v>10% — ideation</v>
       </c>
       <c r="S10" t="str">
-        <v>2024-07-01</v>
+        <v/>
       </c>
       <c r="T10" t="str">
-        <v>2024-08-15</v>
+        <v/>
       </c>
       <c r="U10" t="str">
-        <v>2024-08-01</v>
+        <v/>
       </c>
       <c r="V10" t="str">
-        <v>2024-10-31</v>
+        <v/>
       </c>
       <c r="W10" t="str">
-        <v>2024-11-01</v>
+        <v/>
       </c>
       <c r="X10" t="str">
-        <v>2025-01-31</v>
+        <v/>
       </c>
       <c r="Y10" t="str">
-        <v>2025-02-01</v>
+        <v/>
       </c>
       <c r="Z10" t="str">
-        <v>2025-03-15</v>
+        <v/>
       </c>
       <c r="AA10" t="str">
-        <v>2025-03-16</v>
+        <v/>
       </c>
       <c r="AB10" t="str">
-        <v>2025-03-28</v>
+        <v/>
       </c>
       <c r="AC10" t="str">
         <v/>
       </c>
       <c r="AD10" t="str">
-        <v>100% — Live &amp; stable</v>
+        <v/>
+      </c>
+      <c r="AE10" t="str">
+        <v/>
+      </c>
+      <c r="AF10" t="str">
+        <v/>
+      </c>
+      <c r="AG10" t="str">
+        <v/>
+      </c>
+      <c r="AH10" t="str">
+        <v/>
+      </c>
+      <c r="AI10" t="str">
+        <v/>
+      </c>
+      <c r="AJ10" t="str">
+        <v/>
+      </c>
+      <c r="AK10" t="str">
+        <v/>
+      </c>
+      <c r="AL10" t="str">
+        <v/>
+      </c>
+      <c r="AM10" t="str">
+        <v/>
+      </c>
+      <c r="AN10" t="str">
+        <v>10% — ideation</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>MSL-005</v>
+        <v/>
       </c>
       <c r="B11" t="str">
-        <v>Mobile Approval Workflow App</v>
+        <v>AI Dashboard</v>
       </c>
       <c r="C11" t="str">
-        <v>Digital Transformation</v>
+        <v>Regulatory Compliance</v>
       </c>
       <c r="D11" t="str">
-        <v>IT</v>
+        <v>Marketing</v>
       </c>
       <c r="E11" t="str">
-        <v>IL1</v>
+        <v>IL5</v>
       </c>
       <c r="F11" t="str">
         <v>Innovation</v>
       </c>
       <c r="G11" t="str">
-        <v>2026-27</v>
+        <v>2024-25</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-09-30</v>
+        <v>2024-10-12</v>
       </c>
       <c r="I11" t="str">
-        <v/>
+        <v>2024-11-10</v>
       </c>
       <c r="J11">
-        <v>60</v>
-      </c>
-      <c r="K11" t="str">
-        <v/>
-      </c>
-      <c r="L11" t="str">
-        <v/>
+        <v>14</v>
+      </c>
+      <c r="K11">
+        <v>15999</v>
+      </c>
+      <c r="L11">
+        <v>12</v>
       </c>
       <c r="M11">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N11" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="O11" t="str">
         <v>N</v>
@@ -1406,10 +1636,10 @@
         <v>N</v>
       </c>
       <c r="R11" t="str">
-        <v>10% — ideation</v>
+        <v>It is in progress</v>
       </c>
       <c r="S11" t="str">
-        <v>2026-04-01</v>
+        <v/>
       </c>
       <c r="T11" t="str">
         <v/>
@@ -1442,7 +1672,37 @@
         <v/>
       </c>
       <c r="AD11" t="str">
-        <v>10% — ideation</v>
+        <v/>
+      </c>
+      <c r="AE11" t="str">
+        <v/>
+      </c>
+      <c r="AF11" t="str">
+        <v/>
+      </c>
+      <c r="AG11" t="str">
+        <v/>
+      </c>
+      <c r="AH11" t="str">
+        <v/>
+      </c>
+      <c r="AI11" t="str">
+        <v/>
+      </c>
+      <c r="AJ11" t="str">
+        <v/>
+      </c>
+      <c r="AK11" t="str">
+        <v/>
+      </c>
+      <c r="AL11" t="str">
+        <v/>
+      </c>
+      <c r="AM11" t="str">
+        <v/>
+      </c>
+      <c r="AN11" t="str">
+        <v>It is in progress</v>
       </c>
     </row>
     <row r="12">
@@ -1450,55 +1710,55 @@
         <v/>
       </c>
       <c r="B12" t="str">
-        <v>AI Dashboard</v>
+        <v>AI DASH</v>
       </c>
       <c r="C12" t="str">
-        <v>Regulatory Compliance</v>
+        <v>Customer Experience</v>
       </c>
       <c r="D12" t="str">
-        <v>Marketing</v>
+        <v>IT</v>
       </c>
       <c r="E12" t="str">
-        <v>IL5</v>
+        <v>Live</v>
       </c>
       <c r="F12" t="str">
-        <v>Innovation</v>
+        <v>Compliance</v>
       </c>
       <c r="G12" t="str">
-        <v>2024-25</v>
+        <v>2026-27</v>
       </c>
       <c r="H12" t="str">
-        <v>2024-10-12</v>
+        <v>2026-08-10</v>
       </c>
       <c r="I12" t="str">
-        <v>2024-11-10</v>
+        <v>2026-06-21</v>
       </c>
       <c r="J12">
-        <v>14</v>
+        <v>120</v>
       </c>
       <c r="K12">
-        <v>15999</v>
+        <v>45000</v>
       </c>
       <c r="L12">
+        <v>38</v>
+      </c>
+      <c r="M12">
         <v>12</v>
-      </c>
-      <c r="M12">
-        <v>4</v>
       </c>
       <c r="N12" t="str">
         <v>Y</v>
       </c>
       <c r="O12" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="P12" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="Q12" t="str">
         <v>N</v>
       </c>
       <c r="R12" t="str">
-        <v>It is in progress</v>
+        <v>Quite able to progress so far</v>
       </c>
       <c r="S12" t="str">
         <v/>
@@ -1534,111 +1794,49 @@
         <v/>
       </c>
       <c r="AD12" t="str">
-        <v>It is in progress</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v/>
-      </c>
-      <c r="B13" t="str">
-        <v>AI DASH</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Customer Experience</v>
-      </c>
-      <c r="D13" t="str">
-        <v>IT</v>
-      </c>
-      <c r="E13" t="str">
-        <v>Live</v>
-      </c>
-      <c r="F13" t="str">
-        <v>Compliance</v>
-      </c>
-      <c r="G13" t="str">
-        <v>2026-27</v>
-      </c>
-      <c r="H13" t="str">
-        <v>2026-08-10</v>
-      </c>
-      <c r="I13" t="str">
-        <v>2026-06-21</v>
-      </c>
-      <c r="J13">
-        <v>120</v>
-      </c>
-      <c r="K13">
-        <v>45000</v>
-      </c>
-      <c r="L13">
-        <v>38</v>
-      </c>
-      <c r="M13">
-        <v>12</v>
-      </c>
-      <c r="N13" t="str">
-        <v>Y</v>
-      </c>
-      <c r="O13" t="str">
-        <v>Y</v>
-      </c>
-      <c r="P13" t="str">
-        <v>Y</v>
-      </c>
-      <c r="Q13" t="str">
-        <v>N</v>
-      </c>
-      <c r="R13" t="str">
-        <v>Quite able to progress so far</v>
-      </c>
-      <c r="S13" t="str">
-        <v/>
-      </c>
-      <c r="T13" t="str">
-        <v/>
-      </c>
-      <c r="U13" t="str">
-        <v/>
-      </c>
-      <c r="V13" t="str">
-        <v/>
-      </c>
-      <c r="W13" t="str">
-        <v/>
-      </c>
-      <c r="X13" t="str">
-        <v/>
-      </c>
-      <c r="Y13" t="str">
-        <v/>
-      </c>
-      <c r="Z13" t="str">
-        <v/>
-      </c>
-      <c r="AA13" t="str">
-        <v/>
-      </c>
-      <c r="AB13" t="str">
-        <v/>
-      </c>
-      <c r="AC13" t="str">
-        <v/>
-      </c>
-      <c r="AD13" t="str">
+        <v/>
+      </c>
+      <c r="AE12" t="str">
+        <v/>
+      </c>
+      <c r="AF12" t="str">
+        <v/>
+      </c>
+      <c r="AG12" t="str">
+        <v/>
+      </c>
+      <c r="AH12" t="str">
+        <v/>
+      </c>
+      <c r="AI12" t="str">
+        <v/>
+      </c>
+      <c r="AJ12" t="str">
+        <v/>
+      </c>
+      <c r="AK12" t="str">
+        <v/>
+      </c>
+      <c r="AL12" t="str">
+        <v/>
+      </c>
+      <c r="AM12" t="str">
+        <v/>
+      </c>
+      <c r="AN12" t="str">
         <v>Quite able to progress so far</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN12"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D31"/>
+  <dimension ref="A1:D41"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -1914,24 +2112,24 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>IL1 Phase Start</v>
+        <v>IL1 Target Start</v>
       </c>
       <c r="B20" t="str">
-        <v>il1_start</v>
+        <v>IL1 Target Start</v>
       </c>
       <c r="C20" t="str">
         <v>Gantt Chart</v>
       </c>
       <c r="D20" t="str">
-        <v>2024-04-01  (YYYY-MM-DD)</v>
+        <v>2024-04-01</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>IL1 Phase End</v>
+        <v>IL1 Target End</v>
       </c>
       <c r="B21" t="str">
-        <v>il1_end</v>
+        <v>IL1 Target End</v>
       </c>
       <c r="C21" t="str">
         <v>Gantt Chart</v>
@@ -1942,154 +2140,294 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>IL2 Phase Start</v>
+        <v>IL1 Actual Start</v>
       </c>
       <c r="B22" t="str">
-        <v>il2_start</v>
+        <v>IL1 Actual Start</v>
       </c>
       <c r="C22" t="str">
         <v>Gantt Chart</v>
       </c>
       <c r="D22" t="str">
-        <v>2024-05-01</v>
+        <v>2024-04-05</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>IL2 Phase End</v>
+        <v>IL1 Actual End</v>
       </c>
       <c r="B23" t="str">
-        <v>il2_end</v>
+        <v>IL1 Actual End</v>
       </c>
       <c r="C23" t="str">
         <v>Gantt Chart</v>
       </c>
       <c r="D23" t="str">
-        <v>2024-07-30</v>
+        <v>2024-05-20</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>IL3 Phase Start</v>
+        <v>IL2 Target Start</v>
       </c>
       <c r="B24" t="str">
-        <v>il3_start</v>
+        <v>IL2 Target Start</v>
       </c>
       <c r="C24" t="str">
         <v>Gantt Chart</v>
       </c>
       <c r="D24" t="str">
-        <v>2024-08-01</v>
+        <v>2024-05-01</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>IL3 Phase End</v>
+        <v>IL2 Target End</v>
       </c>
       <c r="B25" t="str">
-        <v>il3_end</v>
+        <v>IL2 Target End</v>
       </c>
       <c r="C25" t="str">
         <v>Gantt Chart</v>
       </c>
       <c r="D25" t="str">
-        <v>2024-11-30</v>
+        <v>2024-07-30</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>IL4 Phase Start</v>
+        <v>IL2 Actual Start</v>
       </c>
       <c r="B26" t="str">
-        <v>il4_start</v>
+        <v>IL2 Actual Start</v>
       </c>
       <c r="C26" t="str">
         <v>Gantt Chart</v>
       </c>
       <c r="D26" t="str">
-        <v>2024-12-01</v>
+        <v>2024-05-01</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>IL4 Phase End</v>
+        <v>IL2 Actual End</v>
       </c>
       <c r="B27" t="str">
-        <v>il4_end</v>
+        <v>IL2 Actual End</v>
       </c>
       <c r="C27" t="str">
         <v>Gantt Chart</v>
       </c>
       <c r="D27" t="str">
-        <v>2025-01-31</v>
+        <v>2024-07-30</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>IL5 Phase Start</v>
+        <v>IL3 Target Start</v>
       </c>
       <c r="B28" t="str">
-        <v>il5_start</v>
+        <v>IL3 Target Start</v>
       </c>
       <c r="C28" t="str">
         <v>Gantt Chart</v>
       </c>
       <c r="D28" t="str">
-        <v>2025-02-01</v>
+        <v>2024-08-01</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>IL5 Phase End</v>
+        <v>IL3 Target End</v>
       </c>
       <c r="B29" t="str">
-        <v>il5_end</v>
+        <v>IL3 Target End</v>
       </c>
       <c r="C29" t="str">
         <v>Gantt Chart</v>
       </c>
       <c r="D29" t="str">
-        <v>2025-03-15</v>
+        <v>2024-11-30</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>Assigned To Staff ID</v>
+        <v>IL3 Actual Start</v>
       </c>
       <c r="B30" t="str">
-        <v>assignedStaffId</v>
+        <v>IL3 Actual Start</v>
       </c>
       <c r="C30" t="str">
-        <v>All Views</v>
+        <v>Gantt Chart</v>
       </c>
       <c r="D30" t="str">
-        <v>EMP123</v>
+        <v>2024-08-01</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
+        <v>IL3 Actual End</v>
+      </c>
+      <c r="B31" t="str">
+        <v>IL3 Actual End</v>
+      </c>
+      <c r="C31" t="str">
+        <v>Gantt Chart</v>
+      </c>
+      <c r="D31" t="str">
+        <v>2024-11-30</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>IL4 Target Start</v>
+      </c>
+      <c r="B32" t="str">
+        <v>IL4 Target Start</v>
+      </c>
+      <c r="C32" t="str">
+        <v>Gantt Chart</v>
+      </c>
+      <c r="D32" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>IL4 Target End</v>
+      </c>
+      <c r="B33" t="str">
+        <v>IL4 Target End</v>
+      </c>
+      <c r="C33" t="str">
+        <v>Gantt Chart</v>
+      </c>
+      <c r="D33" t="str">
+        <v>2025-01-31</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>IL4 Actual Start</v>
+      </c>
+      <c r="B34" t="str">
+        <v>IL4 Actual Start</v>
+      </c>
+      <c r="C34" t="str">
+        <v>Gantt Chart</v>
+      </c>
+      <c r="D34" t="str">
+        <v>2024-12-01</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>IL4 Actual End</v>
+      </c>
+      <c r="B35" t="str">
+        <v>IL4 Actual End</v>
+      </c>
+      <c r="C35" t="str">
+        <v>Gantt Chart</v>
+      </c>
+      <c r="D35" t="str">
+        <v>2025-01-31</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>IL5 Target Start</v>
+      </c>
+      <c r="B36" t="str">
+        <v>IL5 Target Start</v>
+      </c>
+      <c r="C36" t="str">
+        <v>Gantt Chart</v>
+      </c>
+      <c r="D36" t="str">
+        <v>2025-02-01</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>IL5 Target End</v>
+      </c>
+      <c r="B37" t="str">
+        <v>IL5 Target End</v>
+      </c>
+      <c r="C37" t="str">
+        <v>Gantt Chart</v>
+      </c>
+      <c r="D37" t="str">
+        <v>2025-03-15</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>IL5 Actual Start</v>
+      </c>
+      <c r="B38" t="str">
+        <v>IL5 Actual Start</v>
+      </c>
+      <c r="C38" t="str">
+        <v>Gantt Chart</v>
+      </c>
+      <c r="D38" t="str">
+        <v>2025-02-01</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>IL5 Actual End</v>
+      </c>
+      <c r="B39" t="str">
+        <v>IL5 Actual End</v>
+      </c>
+      <c r="C39" t="str">
+        <v>Gantt Chart</v>
+      </c>
+      <c r="D39" t="str">
+        <v>2025-03-15</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>Assigned To Staff ID</v>
+      </c>
+      <c r="B40" t="str">
+        <v>assignedStaffId</v>
+      </c>
+      <c r="C40" t="str">
+        <v>All Views</v>
+      </c>
+      <c r="D40" t="str">
+        <v>EMP123</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
         <v>Overall Progress</v>
       </c>
-      <c r="B31" t="str">
+      <c r="B41" t="str">
         <v>overallStatus</v>
       </c>
-      <c r="C31" t="str">
+      <c r="C41" t="str">
         <v>All Views</v>
       </c>
-      <c r="D31" t="str">
+      <c r="D41" t="str">
         <v>90% complete, UAT started</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D31"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D41"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD1"/>
+  <dimension ref="A1:T1"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -2109,18 +2447,8 @@
     <col min="16" max="16" width="16.83203125" customWidth="1"/>
     <col min="17" max="17" width="19.83203125" customWidth="1"/>
     <col min="18" max="18" width="16.83203125" customWidth="1"/>
-    <col min="19" max="19" width="17.83203125" customWidth="1"/>
-    <col min="20" max="20" width="16.83203125" customWidth="1"/>
-    <col min="21" max="21" width="17.83203125" customWidth="1"/>
-    <col min="22" max="22" width="16.83203125" customWidth="1"/>
-    <col min="23" max="23" width="17.83203125" customWidth="1"/>
-    <col min="24" max="24" width="16.83203125" customWidth="1"/>
-    <col min="25" max="25" width="17.83203125" customWidth="1"/>
-    <col min="26" max="26" width="16.83203125" customWidth="1"/>
-    <col min="27" max="27" width="17.83203125" customWidth="1"/>
-    <col min="28" max="28" width="16.83203125" customWidth="1"/>
-    <col min="29" max="29" width="22.83203125" customWidth="1"/>
-    <col min="30" max="30" width="18.83203125" customWidth="1"/>
+    <col min="19" max="19" width="22.83203125" customWidth="1"/>
+    <col min="20" max="20" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2179,45 +2507,15 @@
         <v>Remarks</v>
       </c>
       <c r="S1" t="str">
-        <v>IL1 Phase Start</v>
+        <v>Assigned To Staff ID</v>
       </c>
       <c r="T1" t="str">
-        <v>IL1 Phase End</v>
-      </c>
-      <c r="U1" t="str">
-        <v>IL2 Phase Start</v>
-      </c>
-      <c r="V1" t="str">
-        <v>IL2 Phase End</v>
-      </c>
-      <c r="W1" t="str">
-        <v>IL3 Phase Start</v>
-      </c>
-      <c r="X1" t="str">
-        <v>IL3 Phase End</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>IL4 Phase Start</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>IL4 Phase End</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>IL5 Phase Start</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>IL5 Phase End</v>
-      </c>
-      <c r="AC1" t="str">
-        <v>Assigned To Staff ID</v>
-      </c>
-      <c r="AD1" t="str">
         <v>Overall Progress</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update project code format to QAQD logic
</commit_message>
<xml_diff>
--- a/PMO_Master.xlsx
+++ b/PMO_Master.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN12"/>
+  <dimension ref="A1:AN8"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -487,58 +487,58 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>MSL-002</v>
+        <v>2526QAQD-001</v>
       </c>
       <c r="B2" t="str">
-        <v>SAP HR Module Integration</v>
+        <v>Vendor Portal Digitization</v>
       </c>
       <c r="C2" t="str">
-        <v>Operational Excellence</v>
+        <v>Digital Transformation</v>
       </c>
       <c r="D2" t="str">
-        <v>HR</v>
+        <v>Finance</v>
       </c>
       <c r="E2" t="str">
-        <v>IL2</v>
+        <v>IL3</v>
       </c>
       <c r="F2" t="str">
-        <v>Integration</v>
+        <v>Process Automation</v>
       </c>
       <c r="G2" t="str">
         <v>2025-26</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-03-31</v>
+        <v>2025-12-31</v>
       </c>
       <c r="I2" t="str">
-        <v/>
+        <v>2026-01-12</v>
       </c>
       <c r="J2">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="K2">
-        <v>1200000</v>
-      </c>
-      <c r="L2" t="str">
-        <v/>
+        <v>850000</v>
+      </c>
+      <c r="L2">
+        <v>38</v>
       </c>
       <c r="M2">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Y</v>
+      </c>
+      <c r="P2" t="str">
         <v>N</v>
-      </c>
-      <c r="O2" t="str">
-        <v>N</v>
-      </c>
-      <c r="P2" t="str">
-        <v>Y</v>
       </c>
       <c r="Q2" t="str">
         <v>Y</v>
       </c>
       <c r="R2" t="str">
-        <v>20% complete</v>
+        <v/>
       </c>
       <c r="S2" t="str">
         <v/>
@@ -604,51 +604,51 @@
         <v/>
       </c>
       <c r="AN2" t="str">
-        <v>20% complete</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>MSL-003</v>
+        <v>2526QAQD-002</v>
       </c>
       <c r="B3" t="str">
-        <v>Customer Complaint Analytics</v>
+        <v>SAP HR Module Integration</v>
       </c>
       <c r="C3" t="str">
-        <v>Customer Experience</v>
+        <v>Operational Excellence</v>
       </c>
       <c r="D3" t="str">
-        <v>Customer Service</v>
+        <v>HR</v>
       </c>
       <c r="E3" t="str">
-        <v>IL4</v>
+        <v>IL2</v>
       </c>
       <c r="F3" t="str">
-        <v>Analytics</v>
+        <v>Integration</v>
       </c>
       <c r="G3" t="str">
-        <v>2024-25</v>
+        <v>2025-26</v>
       </c>
       <c r="H3" t="str">
-        <v>2025-06-30</v>
+        <v>2026-03-31</v>
       </c>
       <c r="I3" t="str">
-        <v>2025-07-15</v>
+        <v/>
       </c>
       <c r="J3">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="K3">
-        <v>340000</v>
-      </c>
-      <c r="L3">
-        <v>55</v>
+        <v>1200000</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
       </c>
       <c r="M3">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="N3" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="O3" t="str">
         <v>N</v>
@@ -660,7 +660,7 @@
         <v>Y</v>
       </c>
       <c r="R3" t="str">
-        <v>95% — live this week</v>
+        <v/>
       </c>
       <c r="S3" t="str">
         <v/>
@@ -726,63 +726,63 @@
         <v/>
       </c>
       <c r="AN3" t="str">
-        <v>95% — live this week</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>MSL-005</v>
+        <v>2425QAQD-001</v>
       </c>
       <c r="B4" t="str">
-        <v>Mobile Approval Workflow App</v>
+        <v>Customer Complaint Analytics</v>
       </c>
       <c r="C4" t="str">
-        <v>Digital Transformation</v>
+        <v>Customer Experience</v>
       </c>
       <c r="D4" t="str">
-        <v>IT</v>
+        <v>Customer Service</v>
       </c>
       <c r="E4" t="str">
-        <v>IL1</v>
+        <v>IL4</v>
       </c>
       <c r="F4" t="str">
-        <v>Innovation</v>
+        <v>Analytics</v>
       </c>
       <c r="G4" t="str">
-        <v>2026-27</v>
+        <v>2024-25</v>
       </c>
       <c r="H4" t="str">
-        <v>2026-09-30</v>
+        <v>2025-06-30</v>
       </c>
       <c r="I4" t="str">
-        <v/>
+        <v>2025-07-15</v>
       </c>
       <c r="J4">
-        <v>60</v>
-      </c>
-      <c r="K4" t="str">
-        <v/>
-      </c>
-      <c r="L4" t="str">
-        <v/>
+        <v>80</v>
+      </c>
+      <c r="K4">
+        <v>340000</v>
+      </c>
+      <c r="L4">
+        <v>55</v>
       </c>
       <c r="M4">
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="N4" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="O4" t="str">
         <v>N</v>
       </c>
       <c r="P4" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="Q4" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="R4" t="str">
-        <v>10% — ideation</v>
+        <v/>
       </c>
       <c r="S4" t="str">
         <v/>
@@ -848,12 +848,12 @@
         <v/>
       </c>
       <c r="AN4" t="str">
-        <v>10% — ideation</v>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>MSL-004</v>
+        <v>2425QAQD-002</v>
       </c>
       <c r="B5" t="str">
         <v>Supply Chain Visibility Dashboard</v>
@@ -904,16 +904,16 @@
         <v>N</v>
       </c>
       <c r="R5" t="str">
-        <v>100% — Live &amp; stable</v>
+        <v/>
       </c>
       <c r="S5" t="str">
-        <v>2024-02-15</v>
+        <v/>
       </c>
       <c r="T5" t="str">
         <v/>
       </c>
       <c r="U5" t="str">
-        <v>2024-06-13</v>
+        <v/>
       </c>
       <c r="V5" t="str">
         <v/>
@@ -970,63 +970,63 @@
         <v/>
       </c>
       <c r="AN5" t="str">
-        <v>100% — Live &amp; stable</v>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>MSL-001</v>
+        <v>2627QAQD-001</v>
       </c>
       <c r="B6" t="str">
-        <v>Vendor Portal Digitization</v>
+        <v>Mobile Approval Workflow App</v>
       </c>
       <c r="C6" t="str">
         <v>Digital Transformation</v>
       </c>
       <c r="D6" t="str">
-        <v>Finance</v>
+        <v>IT</v>
       </c>
       <c r="E6" t="str">
-        <v>IL3</v>
+        <v>IL1</v>
       </c>
       <c r="F6" t="str">
-        <v>Process Automation</v>
+        <v>Innovation</v>
       </c>
       <c r="G6" t="str">
-        <v>2025-26</v>
+        <v>2026-27</v>
       </c>
       <c r="H6" t="str">
-        <v>2025-12-31</v>
+        <v>2026-09-30</v>
       </c>
       <c r="I6" t="str">
-        <v>2026-01-12</v>
+        <v/>
       </c>
       <c r="J6">
-        <v>160</v>
-      </c>
-      <c r="K6">
-        <v>850000</v>
-      </c>
-      <c r="L6">
-        <v>38</v>
+        <v>60</v>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
       </c>
       <c r="M6">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N6" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="O6" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="P6" t="str">
         <v>N</v>
       </c>
       <c r="Q6" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="R6" t="str">
-        <v>65% complete</v>
+        <v/>
       </c>
       <c r="S6" t="str">
         <v/>
@@ -1092,63 +1092,63 @@
         <v/>
       </c>
       <c r="AN6" t="str">
-        <v>65% complete</v>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>MSL-002</v>
+        <v>2425QAQD-003</v>
       </c>
       <c r="B7" t="str">
-        <v>SAP HR Module Integration</v>
+        <v>AI Dashboard</v>
       </c>
       <c r="C7" t="str">
-        <v>Operational Excellence</v>
+        <v>Regulatory Compliance</v>
       </c>
       <c r="D7" t="str">
-        <v>HR</v>
+        <v>Marketing</v>
       </c>
       <c r="E7" t="str">
-        <v>IL2</v>
+        <v>IL5</v>
       </c>
       <c r="F7" t="str">
-        <v>Integration</v>
+        <v>Innovation</v>
       </c>
       <c r="G7" t="str">
-        <v>2025-26</v>
+        <v>2024-25</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-03-31</v>
+        <v>2024-10-12</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>2024-11-10</v>
       </c>
       <c r="J7">
-        <v>120</v>
+        <v>14</v>
       </c>
       <c r="K7">
-        <v>1200000</v>
-      </c>
-      <c r="L7" t="str">
-        <v/>
+        <v>15999</v>
+      </c>
+      <c r="L7">
+        <v>12</v>
       </c>
       <c r="M7">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="N7" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="O7" t="str">
         <v>N</v>
       </c>
       <c r="P7" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="Q7" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="R7" t="str">
-        <v>20% complete</v>
+        <v/>
       </c>
       <c r="S7" t="str">
         <v/>
@@ -1214,63 +1214,63 @@
         <v/>
       </c>
       <c r="AN7" t="str">
-        <v>20% complete</v>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>MSL-003</v>
+        <v>2627QAQD-002</v>
       </c>
       <c r="B8" t="str">
-        <v>Customer Complaint Analytics</v>
+        <v>AI DASH</v>
       </c>
       <c r="C8" t="str">
         <v>Customer Experience</v>
       </c>
       <c r="D8" t="str">
-        <v>Customer Service</v>
+        <v>IT</v>
       </c>
       <c r="E8" t="str">
-        <v>IL4</v>
+        <v>Live</v>
       </c>
       <c r="F8" t="str">
-        <v>Analytics</v>
+        <v>Compliance</v>
       </c>
       <c r="G8" t="str">
-        <v>2024-25</v>
+        <v>2026-27</v>
       </c>
       <c r="H8" t="str">
-        <v>2025-06-30</v>
+        <v>2026-08-10</v>
       </c>
       <c r="I8" t="str">
-        <v>2025-07-15</v>
+        <v>2026-06-21</v>
       </c>
       <c r="J8">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="K8">
-        <v>340000</v>
+        <v>45000</v>
       </c>
       <c r="L8">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="M8">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="N8" t="str">
         <v>Y</v>
       </c>
       <c r="O8" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="P8" t="str">
         <v>Y</v>
       </c>
       <c r="Q8" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="R8" t="str">
-        <v>95% — live this week</v>
+        <v/>
       </c>
       <c r="S8" t="str">
         <v/>
@@ -1336,500 +1336,12 @@
         <v/>
       </c>
       <c r="AN8" t="str">
-        <v>95% — live this week</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>MSL-004</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Supply Chain Visibility Dashboard</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Data &amp; Analytics</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Supply Chain</v>
-      </c>
-      <c r="E9" t="str">
-        <v>Live</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Reporting</v>
-      </c>
-      <c r="G9" t="str">
-        <v>2024-25</v>
-      </c>
-      <c r="H9" t="str">
-        <v>2025-03-31</v>
-      </c>
-      <c r="I9" t="str">
-        <v>2025-03-28</v>
-      </c>
-      <c r="J9">
-        <v>200</v>
-      </c>
-      <c r="K9">
-        <v>675000</v>
-      </c>
-      <c r="L9">
-        <v>72</v>
-      </c>
-      <c r="M9">
-        <v>24</v>
-      </c>
-      <c r="N9" t="str">
-        <v>Y</v>
-      </c>
-      <c r="O9" t="str">
-        <v>Y</v>
-      </c>
-      <c r="P9" t="str">
-        <v>Y</v>
-      </c>
-      <c r="Q9" t="str">
-        <v>N</v>
-      </c>
-      <c r="R9" t="str">
-        <v>100% — Live &amp; stable</v>
-      </c>
-      <c r="S9" t="str">
-        <v/>
-      </c>
-      <c r="T9" t="str">
-        <v/>
-      </c>
-      <c r="U9" t="str">
-        <v/>
-      </c>
-      <c r="V9" t="str">
-        <v/>
-      </c>
-      <c r="W9" t="str">
-        <v/>
-      </c>
-      <c r="X9" t="str">
-        <v/>
-      </c>
-      <c r="Y9" t="str">
-        <v/>
-      </c>
-      <c r="Z9" t="str">
-        <v/>
-      </c>
-      <c r="AA9" t="str">
-        <v/>
-      </c>
-      <c r="AB9" t="str">
-        <v/>
-      </c>
-      <c r="AC9" t="str">
-        <v/>
-      </c>
-      <c r="AD9" t="str">
-        <v/>
-      </c>
-      <c r="AE9" t="str">
-        <v/>
-      </c>
-      <c r="AF9" t="str">
-        <v/>
-      </c>
-      <c r="AG9" t="str">
-        <v/>
-      </c>
-      <c r="AH9" t="str">
-        <v/>
-      </c>
-      <c r="AI9" t="str">
-        <v/>
-      </c>
-      <c r="AJ9" t="str">
-        <v/>
-      </c>
-      <c r="AK9" t="str">
-        <v/>
-      </c>
-      <c r="AL9" t="str">
-        <v/>
-      </c>
-      <c r="AM9" t="str">
-        <v/>
-      </c>
-      <c r="AN9" t="str">
-        <v>100% — Live &amp; stable</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>MSL-005</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Mobile Approval Workflow App</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Digital Transformation</v>
-      </c>
-      <c r="D10" t="str">
-        <v>IT</v>
-      </c>
-      <c r="E10" t="str">
-        <v>IL1</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Innovation</v>
-      </c>
-      <c r="G10" t="str">
-        <v>2026-27</v>
-      </c>
-      <c r="H10" t="str">
-        <v>2026-09-30</v>
-      </c>
-      <c r="I10" t="str">
-        <v/>
-      </c>
-      <c r="J10">
-        <v>60</v>
-      </c>
-      <c r="K10" t="str">
-        <v/>
-      </c>
-      <c r="L10" t="str">
-        <v/>
-      </c>
-      <c r="M10">
-        <v>5</v>
-      </c>
-      <c r="N10" t="str">
-        <v>N</v>
-      </c>
-      <c r="O10" t="str">
-        <v>N</v>
-      </c>
-      <c r="P10" t="str">
-        <v>N</v>
-      </c>
-      <c r="Q10" t="str">
-        <v>N</v>
-      </c>
-      <c r="R10" t="str">
-        <v>10% — ideation</v>
-      </c>
-      <c r="S10" t="str">
-        <v/>
-      </c>
-      <c r="T10" t="str">
-        <v/>
-      </c>
-      <c r="U10" t="str">
-        <v/>
-      </c>
-      <c r="V10" t="str">
-        <v/>
-      </c>
-      <c r="W10" t="str">
-        <v/>
-      </c>
-      <c r="X10" t="str">
-        <v/>
-      </c>
-      <c r="Y10" t="str">
-        <v/>
-      </c>
-      <c r="Z10" t="str">
-        <v/>
-      </c>
-      <c r="AA10" t="str">
-        <v/>
-      </c>
-      <c r="AB10" t="str">
-        <v/>
-      </c>
-      <c r="AC10" t="str">
-        <v/>
-      </c>
-      <c r="AD10" t="str">
-        <v/>
-      </c>
-      <c r="AE10" t="str">
-        <v/>
-      </c>
-      <c r="AF10" t="str">
-        <v/>
-      </c>
-      <c r="AG10" t="str">
-        <v/>
-      </c>
-      <c r="AH10" t="str">
-        <v/>
-      </c>
-      <c r="AI10" t="str">
-        <v/>
-      </c>
-      <c r="AJ10" t="str">
-        <v/>
-      </c>
-      <c r="AK10" t="str">
-        <v/>
-      </c>
-      <c r="AL10" t="str">
-        <v/>
-      </c>
-      <c r="AM10" t="str">
-        <v/>
-      </c>
-      <c r="AN10" t="str">
-        <v>10% — ideation</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v/>
-      </c>
-      <c r="B11" t="str">
-        <v>AI Dashboard</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Regulatory Compliance</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Marketing</v>
-      </c>
-      <c r="E11" t="str">
-        <v>IL5</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Innovation</v>
-      </c>
-      <c r="G11" t="str">
-        <v>2024-25</v>
-      </c>
-      <c r="H11" t="str">
-        <v>2024-10-12</v>
-      </c>
-      <c r="I11" t="str">
-        <v>2024-11-10</v>
-      </c>
-      <c r="J11">
-        <v>14</v>
-      </c>
-      <c r="K11">
-        <v>15999</v>
-      </c>
-      <c r="L11">
-        <v>12</v>
-      </c>
-      <c r="M11">
-        <v>4</v>
-      </c>
-      <c r="N11" t="str">
-        <v>Y</v>
-      </c>
-      <c r="O11" t="str">
-        <v>N</v>
-      </c>
-      <c r="P11" t="str">
-        <v>N</v>
-      </c>
-      <c r="Q11" t="str">
-        <v>N</v>
-      </c>
-      <c r="R11" t="str">
-        <v>It is in progress</v>
-      </c>
-      <c r="S11" t="str">
-        <v/>
-      </c>
-      <c r="T11" t="str">
-        <v/>
-      </c>
-      <c r="U11" t="str">
-        <v/>
-      </c>
-      <c r="V11" t="str">
-        <v/>
-      </c>
-      <c r="W11" t="str">
-        <v/>
-      </c>
-      <c r="X11" t="str">
-        <v/>
-      </c>
-      <c r="Y11" t="str">
-        <v/>
-      </c>
-      <c r="Z11" t="str">
-        <v/>
-      </c>
-      <c r="AA11" t="str">
-        <v/>
-      </c>
-      <c r="AB11" t="str">
-        <v/>
-      </c>
-      <c r="AC11" t="str">
-        <v/>
-      </c>
-      <c r="AD11" t="str">
-        <v/>
-      </c>
-      <c r="AE11" t="str">
-        <v/>
-      </c>
-      <c r="AF11" t="str">
-        <v/>
-      </c>
-      <c r="AG11" t="str">
-        <v/>
-      </c>
-      <c r="AH11" t="str">
-        <v/>
-      </c>
-      <c r="AI11" t="str">
-        <v/>
-      </c>
-      <c r="AJ11" t="str">
-        <v/>
-      </c>
-      <c r="AK11" t="str">
-        <v/>
-      </c>
-      <c r="AL11" t="str">
-        <v/>
-      </c>
-      <c r="AM11" t="str">
-        <v/>
-      </c>
-      <c r="AN11" t="str">
-        <v>It is in progress</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v/>
-      </c>
-      <c r="B12" t="str">
-        <v>AI DASH</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Customer Experience</v>
-      </c>
-      <c r="D12" t="str">
-        <v>IT</v>
-      </c>
-      <c r="E12" t="str">
-        <v>Live</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Compliance</v>
-      </c>
-      <c r="G12" t="str">
-        <v>2026-27</v>
-      </c>
-      <c r="H12" t="str">
-        <v>2026-08-10</v>
-      </c>
-      <c r="I12" t="str">
-        <v>2026-06-21</v>
-      </c>
-      <c r="J12">
-        <v>120</v>
-      </c>
-      <c r="K12">
-        <v>45000</v>
-      </c>
-      <c r="L12">
-        <v>38</v>
-      </c>
-      <c r="M12">
-        <v>12</v>
-      </c>
-      <c r="N12" t="str">
-        <v>Y</v>
-      </c>
-      <c r="O12" t="str">
-        <v>Y</v>
-      </c>
-      <c r="P12" t="str">
-        <v>Y</v>
-      </c>
-      <c r="Q12" t="str">
-        <v>N</v>
-      </c>
-      <c r="R12" t="str">
-        <v>Quite able to progress so far</v>
-      </c>
-      <c r="S12" t="str">
-        <v/>
-      </c>
-      <c r="T12" t="str">
-        <v/>
-      </c>
-      <c r="U12" t="str">
-        <v/>
-      </c>
-      <c r="V12" t="str">
-        <v/>
-      </c>
-      <c r="W12" t="str">
-        <v/>
-      </c>
-      <c r="X12" t="str">
-        <v/>
-      </c>
-      <c r="Y12" t="str">
-        <v/>
-      </c>
-      <c r="Z12" t="str">
-        <v/>
-      </c>
-      <c r="AA12" t="str">
-        <v/>
-      </c>
-      <c r="AB12" t="str">
-        <v/>
-      </c>
-      <c r="AC12" t="str">
-        <v/>
-      </c>
-      <c r="AD12" t="str">
-        <v/>
-      </c>
-      <c r="AE12" t="str">
-        <v/>
-      </c>
-      <c r="AF12" t="str">
-        <v/>
-      </c>
-      <c r="AG12" t="str">
-        <v/>
-      </c>
-      <c r="AH12" t="str">
-        <v/>
-      </c>
-      <c r="AI12" t="str">
-        <v/>
-      </c>
-      <c r="AJ12" t="str">
-        <v/>
-      </c>
-      <c r="AK12" t="str">
-        <v/>
-      </c>
-      <c r="AL12" t="str">
-        <v/>
-      </c>
-      <c r="AM12" t="str">
-        <v/>
-      </c>
-      <c r="AN12" t="str">
-        <v>Quite able to progress so far</v>
+        <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AN8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add hidden legacy parent/child columns to Master Excel for backward compatibility
</commit_message>
<xml_diff>
--- a/PMO_Master.xlsx
+++ b/PMO_Master.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AN8"/>
+  <dimension ref="A1:AS8"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -421,6 +421,11 @@
     <col min="18" max="18" width="16.83203125" customWidth="1"/>
     <col min="19" max="19" width="22.83203125" customWidth="1"/>
     <col min="20" max="20" width="18.83203125" customWidth="1"/>
+    <col min="21" max="21" hidden="true"/>
+    <col min="22" max="22" hidden="true"/>
+    <col min="23" max="23" hidden="true"/>
+    <col min="24" max="24" hidden="true"/>
+    <col min="25" max="25" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -484,6 +489,21 @@
       <c r="T1" t="str">
         <v>Overall Progress</v>
       </c>
+      <c r="U1" t="str">
+        <v>Project Type</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Parent code</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Child C</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Linked Parent code</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>Project family code</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -606,6 +626,21 @@
       <c r="AN2" t="str">
         <v/>
       </c>
+      <c r="AO2" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP2" t="str">
+        <v>2526QAQD-001</v>
+      </c>
+      <c r="AQ2" t="str">
+        <v/>
+      </c>
+      <c r="AR2" t="str">
+        <v/>
+      </c>
+      <c r="AS2" t="str">
+        <v>2526QAQD-001</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -728,6 +763,21 @@
       <c r="AN3" t="str">
         <v/>
       </c>
+      <c r="AO3" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP3" t="str">
+        <v>2526QAQD-002</v>
+      </c>
+      <c r="AQ3" t="str">
+        <v/>
+      </c>
+      <c r="AR3" t="str">
+        <v/>
+      </c>
+      <c r="AS3" t="str">
+        <v>2526QAQD-002</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -850,6 +900,21 @@
       <c r="AN4" t="str">
         <v/>
       </c>
+      <c r="AO4" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP4" t="str">
+        <v>2425QAQD-001</v>
+      </c>
+      <c r="AQ4" t="str">
+        <v/>
+      </c>
+      <c r="AR4" t="str">
+        <v/>
+      </c>
+      <c r="AS4" t="str">
+        <v>2425QAQD-001</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -972,6 +1037,21 @@
       <c r="AN5" t="str">
         <v/>
       </c>
+      <c r="AO5" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP5" t="str">
+        <v>2425QAQD-002</v>
+      </c>
+      <c r="AQ5" t="str">
+        <v/>
+      </c>
+      <c r="AR5" t="str">
+        <v/>
+      </c>
+      <c r="AS5" t="str">
+        <v>2425QAQD-002</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -1094,6 +1174,21 @@
       <c r="AN6" t="str">
         <v/>
       </c>
+      <c r="AO6" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP6" t="str">
+        <v>2627QAQD-001</v>
+      </c>
+      <c r="AQ6" t="str">
+        <v/>
+      </c>
+      <c r="AR6" t="str">
+        <v/>
+      </c>
+      <c r="AS6" t="str">
+        <v>2627QAQD-001</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -1216,6 +1311,21 @@
       <c r="AN7" t="str">
         <v/>
       </c>
+      <c r="AO7" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP7" t="str">
+        <v>2425QAQD-003</v>
+      </c>
+      <c r="AQ7" t="str">
+        <v/>
+      </c>
+      <c r="AR7" t="str">
+        <v/>
+      </c>
+      <c r="AS7" t="str">
+        <v>2425QAQD-003</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -1338,10 +1448,25 @@
       <c r="AN8" t="str">
         <v/>
       </c>
+      <c r="AO8" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP8" t="str">
+        <v>2627QAQD-002</v>
+      </c>
+      <c r="AQ8" t="str">
+        <v/>
+      </c>
+      <c r="AR8" t="str">
+        <v/>
+      </c>
+      <c r="AS8" t="str">
+        <v>2627QAQD-002</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AN8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS8"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1939,7 +2064,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:Y1"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1961,6 +2086,11 @@
     <col min="18" max="18" width="16.83203125" customWidth="1"/>
     <col min="19" max="19" width="22.83203125" customWidth="1"/>
     <col min="20" max="20" width="18.83203125" customWidth="1"/>
+    <col min="21" max="21" width="16.83203125" customWidth="1"/>
+    <col min="22" max="22" width="16.83203125" customWidth="1"/>
+    <col min="23" max="23" width="16.83203125" customWidth="1"/>
+    <col min="24" max="24" width="20.83203125" customWidth="1"/>
+    <col min="25" max="25" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2024,10 +2154,25 @@
       <c r="T1" t="str">
         <v>Overall Progress</v>
       </c>
+      <c r="U1" t="str">
+        <v>Project Type</v>
+      </c>
+      <c r="V1" t="str">
+        <v>Parent code</v>
+      </c>
+      <c r="W1" t="str">
+        <v>Child C</v>
+      </c>
+      <c r="X1" t="str">
+        <v>Linked Parent code</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>Project family code</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix Excel import wiping phase dates and add QAQD generation for imported projects
</commit_message>
<xml_diff>
--- a/PMO_Master.xlsx
+++ b/PMO_Master.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS8"/>
+  <dimension ref="A1:AS11"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -507,58 +507,58 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2526QAQD-001</v>
+        <v/>
       </c>
       <c r="B2" t="str">
-        <v>Vendor Portal Digitization</v>
+        <v>Test Import Project Alpha</v>
       </c>
       <c r="C2" t="str">
-        <v>Digital Transformation</v>
+        <v>Optimization</v>
       </c>
       <c r="D2" t="str">
-        <v>Finance</v>
+        <v>IT</v>
       </c>
       <c r="E2" t="str">
-        <v>IL3</v>
+        <v>IL2</v>
       </c>
       <c r="F2" t="str">
-        <v>Process Automation</v>
+        <v>Dashboard</v>
       </c>
       <c r="G2" t="str">
-        <v>2025-26</v>
+        <v>2026-27</v>
       </c>
       <c r="H2" t="str">
-        <v>2025-12-31</v>
+        <v>2026-12-01</v>
       </c>
       <c r="I2" t="str">
-        <v>2026-01-12</v>
+        <v/>
       </c>
       <c r="J2">
-        <v>160</v>
+        <v>500</v>
       </c>
       <c r="K2">
-        <v>850000</v>
+        <v>150000</v>
       </c>
       <c r="L2">
-        <v>38</v>
+        <v>2</v>
       </c>
       <c r="M2">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N2" t="str">
         <v>Y</v>
       </c>
       <c r="O2" t="str">
+        <v>N</v>
+      </c>
+      <c r="P2" t="str">
         <v>Y</v>
       </c>
-      <c r="P2" t="str">
+      <c r="Q2" t="str">
         <v>N</v>
       </c>
-      <c r="Q2" t="str">
-        <v>Y</v>
-      </c>
       <c r="R2" t="str">
-        <v/>
+        <v>20%</v>
       </c>
       <c r="S2" t="str">
         <v/>
@@ -621,16 +621,16 @@
         <v/>
       </c>
       <c r="AM2" t="str">
-        <v/>
+        <v>EMP123</v>
       </c>
       <c r="AN2" t="str">
-        <v/>
+        <v>20%</v>
       </c>
       <c r="AO2" t="str">
         <v>Parent</v>
       </c>
       <c r="AP2" t="str">
-        <v>2526QAQD-001</v>
+        <v/>
       </c>
       <c r="AQ2" t="str">
         <v/>
@@ -639,63 +639,63 @@
         <v/>
       </c>
       <c r="AS2" t="str">
-        <v>2526QAQD-001</v>
+        <v/>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2526QAQD-002</v>
+        <v/>
       </c>
       <c r="B3" t="str">
-        <v>SAP HR Module Integration</v>
+        <v>Test Import Project Beta</v>
       </c>
       <c r="C3" t="str">
-        <v>Operational Excellence</v>
+        <v>Automation</v>
       </c>
       <c r="D3" t="str">
         <v>HR</v>
       </c>
       <c r="E3" t="str">
-        <v>IL2</v>
+        <v>IL3</v>
       </c>
       <c r="F3" t="str">
-        <v>Integration</v>
+        <v>Bots</v>
       </c>
       <c r="G3" t="str">
-        <v>2025-26</v>
+        <v>26-27</v>
       </c>
       <c r="H3" t="str">
-        <v>2026-03-31</v>
+        <v>2027-02-15</v>
       </c>
       <c r="I3" t="str">
         <v/>
       </c>
       <c r="J3">
-        <v>120</v>
+        <v>350</v>
       </c>
       <c r="K3">
-        <v>1200000</v>
-      </c>
-      <c r="L3" t="str">
-        <v/>
+        <v>85000</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
       </c>
       <c r="M3">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="N3" t="str">
         <v>N</v>
       </c>
       <c r="O3" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="P3" t="str">
         <v>Y</v>
       </c>
       <c r="Q3" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="R3" t="str">
-        <v/>
+        <v>45%</v>
       </c>
       <c r="S3" t="str">
         <v/>
@@ -758,16 +758,16 @@
         <v/>
       </c>
       <c r="AM3" t="str">
-        <v/>
+        <v>EMP456</v>
       </c>
       <c r="AN3" t="str">
-        <v/>
+        <v>45%</v>
       </c>
       <c r="AO3" t="str">
         <v>Parent</v>
       </c>
       <c r="AP3" t="str">
-        <v>2526QAQD-002</v>
+        <v/>
       </c>
       <c r="AQ3" t="str">
         <v/>
@@ -776,48 +776,48 @@
         <v/>
       </c>
       <c r="AS3" t="str">
-        <v>2526QAQD-002</v>
+        <v/>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2425QAQD-001</v>
+        <v>2526QAQD-003</v>
       </c>
       <c r="B4" t="str">
-        <v>Customer Complaint Analytics</v>
+        <v>Validation</v>
       </c>
       <c r="C4" t="str">
-        <v>Customer Experience</v>
+        <v>Operational Excellence</v>
       </c>
       <c r="D4" t="str">
-        <v>Customer Service</v>
+        <v>HR</v>
       </c>
       <c r="E4" t="str">
         <v>IL4</v>
       </c>
       <c r="F4" t="str">
-        <v>Analytics</v>
+        <v>Reporting</v>
       </c>
       <c r="G4" t="str">
-        <v>2024-25</v>
+        <v>2025-26</v>
       </c>
       <c r="H4" t="str">
-        <v>2025-06-30</v>
+        <v>2027-10-24</v>
       </c>
       <c r="I4" t="str">
-        <v>2025-07-15</v>
+        <v>2026-02-02</v>
       </c>
       <c r="J4">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="K4">
-        <v>340000</v>
+        <v>15000</v>
       </c>
       <c r="L4">
-        <v>55</v>
+        <v>120</v>
       </c>
       <c r="M4">
-        <v>18</v>
+        <v>1000</v>
       </c>
       <c r="N4" t="str">
         <v>Y</v>
@@ -829,10 +829,10 @@
         <v>Y</v>
       </c>
       <c r="Q4" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="R4" t="str">
-        <v/>
+        <v>It is the main project.</v>
       </c>
       <c r="S4" t="str">
         <v/>
@@ -898,13 +898,13 @@
         <v/>
       </c>
       <c r="AN4" t="str">
-        <v/>
+        <v>It is the main project.</v>
       </c>
       <c r="AO4" t="str">
         <v>Parent</v>
       </c>
       <c r="AP4" t="str">
-        <v>2425QAQD-001</v>
+        <v>2526QAQD-003</v>
       </c>
       <c r="AQ4" t="str">
         <v/>
@@ -913,57 +913,57 @@
         <v/>
       </c>
       <c r="AS4" t="str">
-        <v>2425QAQD-001</v>
+        <v>2526QAQD-003</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2425QAQD-002</v>
+        <v>2627QAQD-001</v>
       </c>
       <c r="B5" t="str">
-        <v>Supply Chain Visibility Dashboard</v>
+        <v>Mobile Approval Workflow App</v>
       </c>
       <c r="C5" t="str">
-        <v>Data &amp; Analytics</v>
+        <v>Digital Transformation</v>
       </c>
       <c r="D5" t="str">
-        <v>Supply Chain</v>
+        <v>IT</v>
       </c>
       <c r="E5" t="str">
-        <v>Live</v>
+        <v>IL1</v>
       </c>
       <c r="F5" t="str">
-        <v>Reporting</v>
+        <v>Innovation</v>
       </c>
       <c r="G5" t="str">
-        <v>2024-25</v>
+        <v>2026-27</v>
       </c>
       <c r="H5" t="str">
-        <v>2025-03-31</v>
+        <v>2026-09-30</v>
       </c>
       <c r="I5" t="str">
-        <v>2025-03-28</v>
+        <v/>
       </c>
       <c r="J5">
-        <v>200</v>
-      </c>
-      <c r="K5">
-        <v>675000</v>
-      </c>
-      <c r="L5">
-        <v>72</v>
+        <v>60</v>
+      </c>
+      <c r="K5" t="str">
+        <v/>
+      </c>
+      <c r="L5" t="str">
+        <v/>
       </c>
       <c r="M5">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="N5" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="O5" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="P5" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="Q5" t="str">
         <v>N</v>
@@ -1041,7 +1041,7 @@
         <v>Parent</v>
       </c>
       <c r="AP5" t="str">
-        <v>2425QAQD-002</v>
+        <v>2627QAQD-001</v>
       </c>
       <c r="AQ5" t="str">
         <v/>
@@ -1050,60 +1050,60 @@
         <v/>
       </c>
       <c r="AS5" t="str">
-        <v>2425QAQD-002</v>
+        <v>2627QAQD-001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2627QAQD-001</v>
+        <v>2526QAQD-001</v>
       </c>
       <c r="B6" t="str">
-        <v>Mobile Approval Workflow App</v>
+        <v>Vendor Portal Digitization</v>
       </c>
       <c r="C6" t="str">
         <v>Digital Transformation</v>
       </c>
       <c r="D6" t="str">
-        <v>IT</v>
+        <v>Finance</v>
       </c>
       <c r="E6" t="str">
-        <v>IL1</v>
+        <v>IL3</v>
       </c>
       <c r="F6" t="str">
-        <v>Innovation</v>
+        <v>Process Automation</v>
       </c>
       <c r="G6" t="str">
-        <v>2026-27</v>
+        <v>2025-26</v>
       </c>
       <c r="H6" t="str">
-        <v>2026-09-30</v>
+        <v>2025-12-31</v>
       </c>
       <c r="I6" t="str">
-        <v/>
+        <v>2026-01-12</v>
       </c>
       <c r="J6">
-        <v>60</v>
-      </c>
-      <c r="K6" t="str">
-        <v/>
-      </c>
-      <c r="L6" t="str">
-        <v/>
+        <v>160</v>
+      </c>
+      <c r="K6">
+        <v>850000</v>
+      </c>
+      <c r="L6">
+        <v>38</v>
       </c>
       <c r="M6">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="N6" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="O6" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="P6" t="str">
         <v>N</v>
       </c>
       <c r="Q6" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="R6" t="str">
         <v/>
@@ -1178,7 +1178,7 @@
         <v>Parent</v>
       </c>
       <c r="AP6" t="str">
-        <v>2627QAQD-001</v>
+        <v>2526QAQD-001</v>
       </c>
       <c r="AQ6" t="str">
         <v/>
@@ -1187,60 +1187,60 @@
         <v/>
       </c>
       <c r="AS6" t="str">
-        <v>2627QAQD-001</v>
+        <v>2526QAQD-001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2425QAQD-003</v>
+        <v>2526QAQD-002</v>
       </c>
       <c r="B7" t="str">
-        <v>AI Dashboard</v>
+        <v>SAP HR Module Integration</v>
       </c>
       <c r="C7" t="str">
-        <v>Regulatory Compliance</v>
+        <v>Operational Excellence</v>
       </c>
       <c r="D7" t="str">
-        <v>Marketing</v>
+        <v>HR</v>
       </c>
       <c r="E7" t="str">
-        <v>IL5</v>
+        <v>IL2</v>
       </c>
       <c r="F7" t="str">
-        <v>Innovation</v>
+        <v>Integration</v>
       </c>
       <c r="G7" t="str">
-        <v>2024-25</v>
+        <v>2025-26</v>
       </c>
       <c r="H7" t="str">
-        <v>2024-10-12</v>
+        <v>2026-03-31</v>
       </c>
       <c r="I7" t="str">
-        <v>2024-11-10</v>
+        <v/>
       </c>
       <c r="J7">
-        <v>14</v>
+        <v>120</v>
       </c>
       <c r="K7">
-        <v>15999</v>
-      </c>
-      <c r="L7">
+        <v>1200000</v>
+      </c>
+      <c r="L7" t="str">
+        <v/>
+      </c>
+      <c r="M7">
         <v>12</v>
       </c>
-      <c r="M7">
-        <v>4</v>
-      </c>
       <c r="N7" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="O7" t="str">
         <v>N</v>
       </c>
       <c r="P7" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="Q7" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="R7" t="str">
         <v/>
@@ -1315,7 +1315,7 @@
         <v>Parent</v>
       </c>
       <c r="AP7" t="str">
-        <v>2425QAQD-003</v>
+        <v>2526QAQD-002</v>
       </c>
       <c r="AQ7" t="str">
         <v/>
@@ -1324,60 +1324,60 @@
         <v/>
       </c>
       <c r="AS7" t="str">
-        <v>2425QAQD-003</v>
+        <v>2526QAQD-002</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2627QAQD-002</v>
+        <v>2425QAQD-001</v>
       </c>
       <c r="B8" t="str">
-        <v>AI DASH</v>
+        <v>Customer Complaint Analytics</v>
       </c>
       <c r="C8" t="str">
         <v>Customer Experience</v>
       </c>
       <c r="D8" t="str">
-        <v>IT</v>
+        <v>Customer Service</v>
       </c>
       <c r="E8" t="str">
-        <v>Live</v>
+        <v>IL4</v>
       </c>
       <c r="F8" t="str">
-        <v>Compliance</v>
+        <v>Analytics</v>
       </c>
       <c r="G8" t="str">
-        <v>2026-27</v>
+        <v>2024-25</v>
       </c>
       <c r="H8" t="str">
-        <v>2026-08-10</v>
+        <v>2025-06-30</v>
       </c>
       <c r="I8" t="str">
-        <v>2026-06-21</v>
+        <v>2025-07-15</v>
       </c>
       <c r="J8">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="K8">
-        <v>45000</v>
+        <v>340000</v>
       </c>
       <c r="L8">
-        <v>38</v>
+        <v>55</v>
       </c>
       <c r="M8">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="N8" t="str">
         <v>Y</v>
       </c>
       <c r="O8" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="P8" t="str">
         <v>Y</v>
       </c>
       <c r="Q8" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="R8" t="str">
         <v/>
@@ -1452,21 +1452,432 @@
         <v>Parent</v>
       </c>
       <c r="AP8" t="str">
+        <v>2425QAQD-001</v>
+      </c>
+      <c r="AQ8" t="str">
+        <v/>
+      </c>
+      <c r="AR8" t="str">
+        <v/>
+      </c>
+      <c r="AS8" t="str">
+        <v>2425QAQD-001</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>2425QAQD-002</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Supply Chain Visibility Dashboard</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Data &amp; Analytics</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Supply Chain</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Live</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Reporting</v>
+      </c>
+      <c r="G9" t="str">
+        <v>2024-25</v>
+      </c>
+      <c r="H9" t="str">
+        <v>2025-03-31</v>
+      </c>
+      <c r="I9" t="str">
+        <v>2025-03-28</v>
+      </c>
+      <c r="J9">
+        <v>200</v>
+      </c>
+      <c r="K9">
+        <v>675000</v>
+      </c>
+      <c r="L9">
+        <v>72</v>
+      </c>
+      <c r="M9">
+        <v>24</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Y</v>
+      </c>
+      <c r="P9" t="str">
+        <v>Y</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>N</v>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+      <c r="X9" t="str">
+        <v/>
+      </c>
+      <c r="Y9" t="str">
+        <v/>
+      </c>
+      <c r="Z9" t="str">
+        <v/>
+      </c>
+      <c r="AA9" t="str">
+        <v/>
+      </c>
+      <c r="AB9" t="str">
+        <v/>
+      </c>
+      <c r="AC9" t="str">
+        <v/>
+      </c>
+      <c r="AD9" t="str">
+        <v/>
+      </c>
+      <c r="AE9" t="str">
+        <v/>
+      </c>
+      <c r="AF9" t="str">
+        <v/>
+      </c>
+      <c r="AG9" t="str">
+        <v/>
+      </c>
+      <c r="AH9" t="str">
+        <v/>
+      </c>
+      <c r="AI9" t="str">
+        <v/>
+      </c>
+      <c r="AJ9" t="str">
+        <v/>
+      </c>
+      <c r="AK9" t="str">
+        <v/>
+      </c>
+      <c r="AL9" t="str">
+        <v/>
+      </c>
+      <c r="AM9" t="str">
+        <v/>
+      </c>
+      <c r="AN9" t="str">
+        <v/>
+      </c>
+      <c r="AO9" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP9" t="str">
+        <v>2425QAQD-002</v>
+      </c>
+      <c r="AQ9" t="str">
+        <v/>
+      </c>
+      <c r="AR9" t="str">
+        <v/>
+      </c>
+      <c r="AS9" t="str">
+        <v>2425QAQD-002</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>2425QAQD-003</v>
+      </c>
+      <c r="B10" t="str">
+        <v>AI Dashboard</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Regulatory Compliance</v>
+      </c>
+      <c r="D10" t="str">
+        <v>Marketing</v>
+      </c>
+      <c r="E10" t="str">
+        <v>IL5</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Innovation</v>
+      </c>
+      <c r="G10" t="str">
+        <v>2024-25</v>
+      </c>
+      <c r="H10" t="str">
+        <v>2024-10-12</v>
+      </c>
+      <c r="I10" t="str">
+        <v>2024-11-10</v>
+      </c>
+      <c r="J10">
+        <v>14</v>
+      </c>
+      <c r="K10">
+        <v>15999</v>
+      </c>
+      <c r="L10">
+        <v>12</v>
+      </c>
+      <c r="M10">
+        <v>4</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O10" t="str">
+        <v>N</v>
+      </c>
+      <c r="P10" t="str">
+        <v>N</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>N</v>
+      </c>
+      <c r="R10" t="str">
+        <v/>
+      </c>
+      <c r="S10" t="str">
+        <v/>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v/>
+      </c>
+      <c r="V10" t="str">
+        <v/>
+      </c>
+      <c r="W10" t="str">
+        <v/>
+      </c>
+      <c r="X10" t="str">
+        <v/>
+      </c>
+      <c r="Y10" t="str">
+        <v/>
+      </c>
+      <c r="Z10" t="str">
+        <v/>
+      </c>
+      <c r="AA10" t="str">
+        <v/>
+      </c>
+      <c r="AB10" t="str">
+        <v/>
+      </c>
+      <c r="AC10" t="str">
+        <v/>
+      </c>
+      <c r="AD10" t="str">
+        <v/>
+      </c>
+      <c r="AE10" t="str">
+        <v/>
+      </c>
+      <c r="AF10" t="str">
+        <v/>
+      </c>
+      <c r="AG10" t="str">
+        <v/>
+      </c>
+      <c r="AH10" t="str">
+        <v/>
+      </c>
+      <c r="AI10" t="str">
+        <v/>
+      </c>
+      <c r="AJ10" t="str">
+        <v/>
+      </c>
+      <c r="AK10" t="str">
+        <v/>
+      </c>
+      <c r="AL10" t="str">
+        <v/>
+      </c>
+      <c r="AM10" t="str">
+        <v/>
+      </c>
+      <c r="AN10" t="str">
+        <v/>
+      </c>
+      <c r="AO10" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP10" t="str">
+        <v>2425QAQD-003</v>
+      </c>
+      <c r="AQ10" t="str">
+        <v/>
+      </c>
+      <c r="AR10" t="str">
+        <v/>
+      </c>
+      <c r="AS10" t="str">
+        <v>2425QAQD-003</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>2627QAQD-002</v>
       </c>
-      <c r="AQ8" t="str">
-        <v/>
-      </c>
-      <c r="AR8" t="str">
-        <v/>
-      </c>
-      <c r="AS8" t="str">
+      <c r="B11" t="str">
+        <v>AI DASH</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Customer Experience</v>
+      </c>
+      <c r="D11" t="str">
+        <v>IT</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Live</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Compliance</v>
+      </c>
+      <c r="G11" t="str">
+        <v>2026-27</v>
+      </c>
+      <c r="H11" t="str">
+        <v>2026-08-10</v>
+      </c>
+      <c r="I11" t="str">
+        <v>2026-06-21</v>
+      </c>
+      <c r="J11">
+        <v>120</v>
+      </c>
+      <c r="K11">
+        <v>45000</v>
+      </c>
+      <c r="L11">
+        <v>38</v>
+      </c>
+      <c r="M11">
+        <v>12</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Y</v>
+      </c>
+      <c r="P11" t="str">
+        <v>Y</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>N</v>
+      </c>
+      <c r="R11" t="str">
+        <v/>
+      </c>
+      <c r="S11" t="str">
+        <v/>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v/>
+      </c>
+      <c r="V11" t="str">
+        <v/>
+      </c>
+      <c r="W11" t="str">
+        <v/>
+      </c>
+      <c r="X11" t="str">
+        <v/>
+      </c>
+      <c r="Y11" t="str">
+        <v/>
+      </c>
+      <c r="Z11" t="str">
+        <v/>
+      </c>
+      <c r="AA11" t="str">
+        <v/>
+      </c>
+      <c r="AB11" t="str">
+        <v/>
+      </c>
+      <c r="AC11" t="str">
+        <v/>
+      </c>
+      <c r="AD11" t="str">
+        <v/>
+      </c>
+      <c r="AE11" t="str">
+        <v/>
+      </c>
+      <c r="AF11" t="str">
+        <v/>
+      </c>
+      <c r="AG11" t="str">
+        <v/>
+      </c>
+      <c r="AH11" t="str">
+        <v/>
+      </c>
+      <c r="AI11" t="str">
+        <v/>
+      </c>
+      <c r="AJ11" t="str">
+        <v/>
+      </c>
+      <c r="AK11" t="str">
+        <v/>
+      </c>
+      <c r="AL11" t="str">
+        <v/>
+      </c>
+      <c r="AM11" t="str">
+        <v/>
+      </c>
+      <c r="AN11" t="str">
+        <v/>
+      </c>
+      <c r="AO11" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP11" t="str">
+        <v>2627QAQD-002</v>
+      </c>
+      <c r="AQ11" t="str">
+        <v/>
+      </c>
+      <c r="AR11" t="str">
+        <v/>
+      </c>
+      <c r="AS11" t="str">
         <v>2627QAQD-002</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS11"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Fix Gantt logic bug incorrectly filtering out projects
</commit_message>
<xml_diff>
--- a/PMO_Master.xlsx
+++ b/PMO_Master.xlsx
@@ -421,11 +421,31 @@
     <col min="18" max="18" width="16.83203125" customWidth="1"/>
     <col min="19" max="19" width="22.83203125" customWidth="1"/>
     <col min="20" max="20" width="18.83203125" customWidth="1"/>
-    <col min="21" max="21" hidden="true"/>
-    <col min="22" max="22" hidden="true"/>
-    <col min="23" max="23" hidden="true"/>
-    <col min="24" max="24" hidden="true"/>
-    <col min="25" max="25" hidden="true"/>
+    <col min="21" max="21" width="18.83203125" customWidth="1"/>
+    <col min="22" max="22" width="16.83203125" customWidth="1"/>
+    <col min="23" max="23" width="18.83203125" customWidth="1"/>
+    <col min="24" max="24" width="16.83203125" customWidth="1"/>
+    <col min="25" max="25" width="18.83203125" customWidth="1"/>
+    <col min="26" max="26" width="16.83203125" customWidth="1"/>
+    <col min="27" max="27" width="18.83203125" customWidth="1"/>
+    <col min="28" max="28" width="16.83203125" customWidth="1"/>
+    <col min="29" max="29" width="18.83203125" customWidth="1"/>
+    <col min="30" max="30" width="16.83203125" customWidth="1"/>
+    <col min="31" max="31" width="18.83203125" customWidth="1"/>
+    <col min="32" max="32" width="16.83203125" customWidth="1"/>
+    <col min="33" max="33" width="18.83203125" customWidth="1"/>
+    <col min="34" max="34" width="16.83203125" customWidth="1"/>
+    <col min="35" max="35" width="18.83203125" customWidth="1"/>
+    <col min="36" max="36" width="16.83203125" customWidth="1"/>
+    <col min="37" max="37" width="18.83203125" customWidth="1"/>
+    <col min="38" max="38" width="16.83203125" customWidth="1"/>
+    <col min="39" max="39" width="18.83203125" customWidth="1"/>
+    <col min="40" max="40" width="16.83203125" customWidth="1"/>
+    <col min="41" max="41" hidden="true"/>
+    <col min="42" max="42" hidden="true"/>
+    <col min="43" max="43" hidden="true"/>
+    <col min="44" max="44" hidden="true"/>
+    <col min="45" max="45" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -490,24 +510,84 @@
         <v>Overall Progress</v>
       </c>
       <c r="U1" t="str">
+        <v>IL1 Target Start</v>
+      </c>
+      <c r="V1" t="str">
+        <v>IL1 Target End</v>
+      </c>
+      <c r="W1" t="str">
+        <v>IL1 Actual Start</v>
+      </c>
+      <c r="X1" t="str">
+        <v>IL1 Actual End</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>IL2 Target Start</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>IL2 Target End</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>IL2 Actual Start</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>IL2 Actual End</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>IL3 Target Start</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>IL3 Target End</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>IL3 Actual Start</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>IL3 Actual End</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>IL4 Target Start</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>IL4 Target End</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>IL4 Actual Start</v>
+      </c>
+      <c r="AJ1" t="str">
+        <v>IL4 Actual End</v>
+      </c>
+      <c r="AK1" t="str">
+        <v>IL5 Target Start</v>
+      </c>
+      <c r="AL1" t="str">
+        <v>IL5 Target End</v>
+      </c>
+      <c r="AM1" t="str">
+        <v>IL5 Actual Start</v>
+      </c>
+      <c r="AN1" t="str">
+        <v>IL5 Actual End</v>
+      </c>
+      <c r="AO1" t="str">
         <v>Project Type</v>
       </c>
-      <c r="V1" t="str">
+      <c r="AP1" t="str">
         <v>Parent code</v>
       </c>
-      <c r="W1" t="str">
+      <c r="AQ1" t="str">
         <v>Child C</v>
       </c>
-      <c r="X1" t="str">
+      <c r="AR1" t="str">
         <v>Linked Parent code</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AS1" t="str">
         <v>Project family code</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v/>
+        <v>2627QAQD-003</v>
       </c>
       <c r="B2" t="str">
         <v>Test Import Project Alpha</v>
@@ -630,7 +710,7 @@
         <v>Parent</v>
       </c>
       <c r="AP2" t="str">
-        <v/>
+        <v>2627QAQD-003</v>
       </c>
       <c r="AQ2" t="str">
         <v/>
@@ -639,12 +719,12 @@
         <v/>
       </c>
       <c r="AS2" t="str">
-        <v/>
+        <v>2627QAQD-003</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v/>
+        <v>2627QAQD-004</v>
       </c>
       <c r="B3" t="str">
         <v>Test Import Project Beta</v>
@@ -767,7 +847,7 @@
         <v>Parent</v>
       </c>
       <c r="AP3" t="str">
-        <v/>
+        <v>2627QAQD-004</v>
       </c>
       <c r="AQ3" t="str">
         <v/>
@@ -776,7 +856,7 @@
         <v/>
       </c>
       <c r="AS3" t="str">
-        <v/>
+        <v>2627QAQD-004</v>
       </c>
     </row>
     <row r="4">
@@ -2475,7 +2555,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y1"/>
+  <dimension ref="A1:AS1"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -2497,11 +2577,31 @@
     <col min="18" max="18" width="16.83203125" customWidth="1"/>
     <col min="19" max="19" width="22.83203125" customWidth="1"/>
     <col min="20" max="20" width="18.83203125" customWidth="1"/>
-    <col min="21" max="21" width="16.83203125" customWidth="1"/>
+    <col min="21" max="21" width="18.83203125" customWidth="1"/>
     <col min="22" max="22" width="16.83203125" customWidth="1"/>
-    <col min="23" max="23" width="16.83203125" customWidth="1"/>
-    <col min="24" max="24" width="20.83203125" customWidth="1"/>
-    <col min="25" max="25" width="21.83203125" customWidth="1"/>
+    <col min="23" max="23" width="18.83203125" customWidth="1"/>
+    <col min="24" max="24" width="16.83203125" customWidth="1"/>
+    <col min="25" max="25" width="18.83203125" customWidth="1"/>
+    <col min="26" max="26" width="16.83203125" customWidth="1"/>
+    <col min="27" max="27" width="18.83203125" customWidth="1"/>
+    <col min="28" max="28" width="16.83203125" customWidth="1"/>
+    <col min="29" max="29" width="18.83203125" customWidth="1"/>
+    <col min="30" max="30" width="16.83203125" customWidth="1"/>
+    <col min="31" max="31" width="18.83203125" customWidth="1"/>
+    <col min="32" max="32" width="16.83203125" customWidth="1"/>
+    <col min="33" max="33" width="18.83203125" customWidth="1"/>
+    <col min="34" max="34" width="16.83203125" customWidth="1"/>
+    <col min="35" max="35" width="18.83203125" customWidth="1"/>
+    <col min="36" max="36" width="16.83203125" customWidth="1"/>
+    <col min="37" max="37" width="18.83203125" customWidth="1"/>
+    <col min="38" max="38" width="16.83203125" customWidth="1"/>
+    <col min="39" max="39" width="18.83203125" customWidth="1"/>
+    <col min="40" max="40" width="16.83203125" customWidth="1"/>
+    <col min="41" max="41" width="16.83203125" customWidth="1"/>
+    <col min="42" max="42" width="16.83203125" customWidth="1"/>
+    <col min="43" max="43" width="16.83203125" customWidth="1"/>
+    <col min="44" max="44" width="20.83203125" customWidth="1"/>
+    <col min="45" max="45" width="21.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2566,24 +2666,84 @@
         <v>Overall Progress</v>
       </c>
       <c r="U1" t="str">
+        <v>IL1 Target Start</v>
+      </c>
+      <c r="V1" t="str">
+        <v>IL1 Target End</v>
+      </c>
+      <c r="W1" t="str">
+        <v>IL1 Actual Start</v>
+      </c>
+      <c r="X1" t="str">
+        <v>IL1 Actual End</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>IL2 Target Start</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>IL2 Target End</v>
+      </c>
+      <c r="AA1" t="str">
+        <v>IL2 Actual Start</v>
+      </c>
+      <c r="AB1" t="str">
+        <v>IL2 Actual End</v>
+      </c>
+      <c r="AC1" t="str">
+        <v>IL3 Target Start</v>
+      </c>
+      <c r="AD1" t="str">
+        <v>IL3 Target End</v>
+      </c>
+      <c r="AE1" t="str">
+        <v>IL3 Actual Start</v>
+      </c>
+      <c r="AF1" t="str">
+        <v>IL3 Actual End</v>
+      </c>
+      <c r="AG1" t="str">
+        <v>IL4 Target Start</v>
+      </c>
+      <c r="AH1" t="str">
+        <v>IL4 Target End</v>
+      </c>
+      <c r="AI1" t="str">
+        <v>IL4 Actual Start</v>
+      </c>
+      <c r="AJ1" t="str">
+        <v>IL4 Actual End</v>
+      </c>
+      <c r="AK1" t="str">
+        <v>IL5 Target Start</v>
+      </c>
+      <c r="AL1" t="str">
+        <v>IL5 Target End</v>
+      </c>
+      <c r="AM1" t="str">
+        <v>IL5 Actual Start</v>
+      </c>
+      <c r="AN1" t="str">
+        <v>IL5 Actual End</v>
+      </c>
+      <c r="AO1" t="str">
         <v>Project Type</v>
       </c>
-      <c r="V1" t="str">
+      <c r="AP1" t="str">
         <v>Parent code</v>
       </c>
-      <c r="W1" t="str">
+      <c r="AQ1" t="str">
         <v>Child C</v>
       </c>
-      <c r="X1" t="str">
+      <c r="AR1" t="str">
         <v>Linked Parent code</v>
       </c>
-      <c r="Y1" t="str">
+      <c r="AS1" t="str">
         <v>Project family code</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Grok AI Chatbot integration
</commit_message>
<xml_diff>
--- a/PMO_Master.xlsx
+++ b/PMO_Master.xlsx
@@ -638,7 +638,7 @@
         <v>N</v>
       </c>
       <c r="R2" t="str">
-        <v>20%</v>
+        <v/>
       </c>
       <c r="S2" t="str">
         <v/>
@@ -701,10 +701,10 @@
         <v/>
       </c>
       <c r="AM2" t="str">
-        <v>EMP123</v>
+        <v/>
       </c>
       <c r="AN2" t="str">
-        <v>20%</v>
+        <v/>
       </c>
       <c r="AO2" t="str">
         <v>Parent</v>
@@ -756,8 +756,8 @@
       <c r="K3">
         <v>85000</v>
       </c>
-      <c r="L3">
-        <v>0</v>
+      <c r="L3" t="str">
+        <v/>
       </c>
       <c r="M3">
         <v>3</v>
@@ -775,7 +775,7 @@
         <v>N</v>
       </c>
       <c r="R3" t="str">
-        <v>45%</v>
+        <v/>
       </c>
       <c r="S3" t="str">
         <v/>
@@ -835,13 +835,13 @@
         <v/>
       </c>
       <c r="AL3" t="str">
-        <v/>
+        <v>2044-12-31</v>
       </c>
       <c r="AM3" t="str">
-        <v>EMP456</v>
+        <v/>
       </c>
       <c r="AN3" t="str">
-        <v>45%</v>
+        <v/>
       </c>
       <c r="AO3" t="str">
         <v>Parent</v>
@@ -915,16 +915,16 @@
         <v>It is the main project.</v>
       </c>
       <c r="S4" t="str">
-        <v/>
+        <v>2027-10-02</v>
       </c>
       <c r="T4" t="str">
-        <v/>
+        <v>2027-11-03</v>
       </c>
       <c r="U4" t="str">
-        <v/>
+        <v>2027-08-02</v>
       </c>
       <c r="V4" t="str">
-        <v/>
+        <v>2027-12-04</v>
       </c>
       <c r="W4" t="str">
         <v/>

</xml_diff>

<commit_message>
Add clear chat button and wipe chat history when switching users
</commit_message>
<xml_diff>
--- a/PMO_Master.xlsx
+++ b/PMO_Master.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AS11"/>
+  <dimension ref="A1:AS12"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -587,52 +587,52 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>2627QAQD-003</v>
+        <v>2425QAQD-004</v>
       </c>
       <c r="B2" t="str">
-        <v>Test Import Project Alpha</v>
+        <v>YesWeDo</v>
       </c>
       <c r="C2" t="str">
-        <v>Optimization</v>
+        <v>Regulatory Compliance</v>
       </c>
       <c r="D2" t="str">
-        <v>IT</v>
+        <v>Marketing</v>
       </c>
       <c r="E2" t="str">
-        <v>IL2</v>
+        <v>Live</v>
       </c>
       <c r="F2" t="str">
-        <v>Dashboard</v>
+        <v>Innovation</v>
       </c>
       <c r="G2" t="str">
-        <v>2026-27</v>
+        <v>2024-25</v>
       </c>
       <c r="H2" t="str">
-        <v>2026-12-01</v>
+        <v/>
       </c>
       <c r="I2" t="str">
         <v/>
       </c>
-      <c r="J2">
-        <v>500</v>
-      </c>
-      <c r="K2">
-        <v>150000</v>
-      </c>
-      <c r="L2">
-        <v>2</v>
-      </c>
-      <c r="M2">
-        <v>5</v>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v/>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
       </c>
       <c r="N2" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="O2" t="str">
         <v>N</v>
       </c>
       <c r="P2" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="Q2" t="str">
         <v>N</v>
@@ -710,7 +710,7 @@
         <v>Parent</v>
       </c>
       <c r="AP2" t="str">
-        <v>2627QAQD-003</v>
+        <v>2425QAQD-004</v>
       </c>
       <c r="AQ2" t="str">
         <v/>
@@ -719,54 +719,54 @@
         <v/>
       </c>
       <c r="AS2" t="str">
-        <v>2627QAQD-003</v>
+        <v>2425QAQD-004</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>2627QAQD-004</v>
+        <v>2627QAQD-003</v>
       </c>
       <c r="B3" t="str">
-        <v>Test Import Project Beta</v>
+        <v>Test Import Project Alpha</v>
       </c>
       <c r="C3" t="str">
-        <v>Automation</v>
+        <v>Optimization</v>
       </c>
       <c r="D3" t="str">
-        <v>HR</v>
+        <v>IT</v>
       </c>
       <c r="E3" t="str">
-        <v>IL3</v>
+        <v>IL2</v>
       </c>
       <c r="F3" t="str">
-        <v>Bots</v>
+        <v>Dashboard</v>
       </c>
       <c r="G3" t="str">
-        <v>26-27</v>
+        <v>2026-27</v>
       </c>
       <c r="H3" t="str">
-        <v>2027-02-15</v>
+        <v>2026-12-01</v>
       </c>
       <c r="I3" t="str">
         <v/>
       </c>
       <c r="J3">
-        <v>350</v>
+        <v>500</v>
       </c>
       <c r="K3">
-        <v>85000</v>
-      </c>
-      <c r="L3" t="str">
-        <v/>
+        <v>150000</v>
+      </c>
+      <c r="L3">
+        <v>2</v>
       </c>
       <c r="M3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N3" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O3" t="str">
         <v>N</v>
-      </c>
-      <c r="O3" t="str">
-        <v>Y</v>
       </c>
       <c r="P3" t="str">
         <v>Y</v>
@@ -835,7 +835,7 @@
         <v/>
       </c>
       <c r="AL3" t="str">
-        <v>2044-12-31</v>
+        <v/>
       </c>
       <c r="AM3" t="str">
         <v/>
@@ -847,7 +847,7 @@
         <v>Parent</v>
       </c>
       <c r="AP3" t="str">
-        <v>2627QAQD-004</v>
+        <v>2627QAQD-003</v>
       </c>
       <c r="AQ3" t="str">
         <v/>
@@ -856,54 +856,54 @@
         <v/>
       </c>
       <c r="AS3" t="str">
-        <v>2627QAQD-004</v>
+        <v>2627QAQD-003</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>2526QAQD-003</v>
+        <v>2627QAQD-004</v>
       </c>
       <c r="B4" t="str">
-        <v>Validation</v>
+        <v>Test Import Project Beta</v>
       </c>
       <c r="C4" t="str">
-        <v>Operational Excellence</v>
+        <v>Automation</v>
       </c>
       <c r="D4" t="str">
         <v>HR</v>
       </c>
       <c r="E4" t="str">
-        <v>IL4</v>
+        <v>IL3</v>
       </c>
       <c r="F4" t="str">
-        <v>Reporting</v>
+        <v>Bots</v>
       </c>
       <c r="G4" t="str">
-        <v>2025-26</v>
+        <v>26-27</v>
       </c>
       <c r="H4" t="str">
-        <v>2027-10-24</v>
+        <v>2027-02-15</v>
       </c>
       <c r="I4" t="str">
-        <v>2026-02-02</v>
+        <v/>
       </c>
       <c r="J4">
-        <v>140</v>
+        <v>350</v>
       </c>
       <c r="K4">
-        <v>15000</v>
-      </c>
-      <c r="L4">
-        <v>120</v>
+        <v>85000</v>
+      </c>
+      <c r="L4" t="str">
+        <v/>
       </c>
       <c r="M4">
-        <v>1000</v>
+        <v>3</v>
       </c>
       <c r="N4" t="str">
+        <v>N</v>
+      </c>
+      <c r="O4" t="str">
         <v>Y</v>
-      </c>
-      <c r="O4" t="str">
-        <v>N</v>
       </c>
       <c r="P4" t="str">
         <v>Y</v>
@@ -912,19 +912,19 @@
         <v>N</v>
       </c>
       <c r="R4" t="str">
-        <v>It is the main project.</v>
+        <v/>
       </c>
       <c r="S4" t="str">
-        <v>2027-10-02</v>
+        <v/>
       </c>
       <c r="T4" t="str">
-        <v>2027-11-03</v>
+        <v/>
       </c>
       <c r="U4" t="str">
-        <v>2027-08-02</v>
+        <v/>
       </c>
       <c r="V4" t="str">
-        <v>2027-12-04</v>
+        <v/>
       </c>
       <c r="W4" t="str">
         <v/>
@@ -972,19 +972,19 @@
         <v/>
       </c>
       <c r="AL4" t="str">
-        <v/>
+        <v>2044-12-31</v>
       </c>
       <c r="AM4" t="str">
         <v/>
       </c>
       <c r="AN4" t="str">
-        <v>It is the main project.</v>
+        <v/>
       </c>
       <c r="AO4" t="str">
         <v>Parent</v>
       </c>
       <c r="AP4" t="str">
-        <v>2526QAQD-003</v>
+        <v>2627QAQD-004</v>
       </c>
       <c r="AQ4" t="str">
         <v/>
@@ -993,75 +993,75 @@
         <v/>
       </c>
       <c r="AS4" t="str">
-        <v>2526QAQD-003</v>
+        <v>2627QAQD-004</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>2627QAQD-001</v>
+        <v>2526QAQD-003</v>
       </c>
       <c r="B5" t="str">
-        <v>Mobile Approval Workflow App</v>
+        <v>Validation</v>
       </c>
       <c r="C5" t="str">
-        <v>Digital Transformation</v>
+        <v>Operational Excellence</v>
       </c>
       <c r="D5" t="str">
-        <v>IT</v>
+        <v>HR</v>
       </c>
       <c r="E5" t="str">
-        <v>IL1</v>
+        <v>IL4</v>
       </c>
       <c r="F5" t="str">
-        <v>Innovation</v>
+        <v>Reporting</v>
       </c>
       <c r="G5" t="str">
-        <v>2026-27</v>
+        <v>2025-26</v>
       </c>
       <c r="H5" t="str">
-        <v>2026-09-30</v>
+        <v>2027-10-24</v>
       </c>
       <c r="I5" t="str">
-        <v/>
+        <v>2026-02-02</v>
       </c>
       <c r="J5">
-        <v>60</v>
-      </c>
-      <c r="K5" t="str">
-        <v/>
-      </c>
-      <c r="L5" t="str">
-        <v/>
+        <v>140</v>
+      </c>
+      <c r="K5">
+        <v>15000</v>
+      </c>
+      <c r="L5">
+        <v>120</v>
       </c>
       <c r="M5">
-        <v>5</v>
+        <v>1000</v>
       </c>
       <c r="N5" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="O5" t="str">
         <v>N</v>
       </c>
       <c r="P5" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="Q5" t="str">
         <v>N</v>
       </c>
       <c r="R5" t="str">
-        <v/>
+        <v>It is the main project.</v>
       </c>
       <c r="S5" t="str">
-        <v/>
+        <v>2027-10-02</v>
       </c>
       <c r="T5" t="str">
-        <v/>
+        <v>2027-11-03</v>
       </c>
       <c r="U5" t="str">
-        <v/>
+        <v>2027-08-02</v>
       </c>
       <c r="V5" t="str">
-        <v/>
+        <v>2027-12-04</v>
       </c>
       <c r="W5" t="str">
         <v/>
@@ -1115,13 +1115,13 @@
         <v/>
       </c>
       <c r="AN5" t="str">
-        <v/>
+        <v>It is the main project.</v>
       </c>
       <c r="AO5" t="str">
         <v>Parent</v>
       </c>
       <c r="AP5" t="str">
-        <v>2627QAQD-001</v>
+        <v>2526QAQD-003</v>
       </c>
       <c r="AQ5" t="str">
         <v/>
@@ -1130,60 +1130,60 @@
         <v/>
       </c>
       <c r="AS5" t="str">
-        <v>2627QAQD-001</v>
+        <v>2526QAQD-003</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>2526QAQD-001</v>
+        <v>2627QAQD-001</v>
       </c>
       <c r="B6" t="str">
-        <v>Vendor Portal Digitization</v>
+        <v>Mobile Approval Workflow App</v>
       </c>
       <c r="C6" t="str">
         <v>Digital Transformation</v>
       </c>
       <c r="D6" t="str">
-        <v>Finance</v>
+        <v>IT</v>
       </c>
       <c r="E6" t="str">
-        <v>IL3</v>
+        <v>IL1</v>
       </c>
       <c r="F6" t="str">
-        <v>Process Automation</v>
+        <v>Innovation</v>
       </c>
       <c r="G6" t="str">
-        <v>2025-26</v>
+        <v>2026-27</v>
       </c>
       <c r="H6" t="str">
-        <v>2025-12-31</v>
+        <v>2026-09-30</v>
       </c>
       <c r="I6" t="str">
-        <v>2026-01-12</v>
+        <v/>
       </c>
       <c r="J6">
-        <v>160</v>
-      </c>
-      <c r="K6">
-        <v>850000</v>
-      </c>
-      <c r="L6">
-        <v>38</v>
+        <v>60</v>
+      </c>
+      <c r="K6" t="str">
+        <v/>
+      </c>
+      <c r="L6" t="str">
+        <v/>
       </c>
       <c r="M6">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="N6" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="O6" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="P6" t="str">
         <v>N</v>
       </c>
       <c r="Q6" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="R6" t="str">
         <v/>
@@ -1258,7 +1258,7 @@
         <v>Parent</v>
       </c>
       <c r="AP6" t="str">
-        <v>2526QAQD-001</v>
+        <v>2627QAQD-001</v>
       </c>
       <c r="AQ6" t="str">
         <v/>
@@ -1267,57 +1267,57 @@
         <v/>
       </c>
       <c r="AS6" t="str">
-        <v>2526QAQD-001</v>
+        <v>2627QAQD-001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>2526QAQD-002</v>
+        <v>2526QAQD-001</v>
       </c>
       <c r="B7" t="str">
-        <v>SAP HR Module Integration</v>
+        <v>Vendor Portal Digitization</v>
       </c>
       <c r="C7" t="str">
-        <v>Operational Excellence</v>
+        <v>Digital Transformation</v>
       </c>
       <c r="D7" t="str">
-        <v>HR</v>
+        <v>Finance</v>
       </c>
       <c r="E7" t="str">
-        <v>IL2</v>
+        <v>IL3</v>
       </c>
       <c r="F7" t="str">
-        <v>Integration</v>
+        <v>Process Automation</v>
       </c>
       <c r="G7" t="str">
         <v>2025-26</v>
       </c>
       <c r="H7" t="str">
-        <v>2026-03-31</v>
+        <v>2025-12-31</v>
       </c>
       <c r="I7" t="str">
-        <v/>
+        <v>2026-01-12</v>
       </c>
       <c r="J7">
-        <v>120</v>
+        <v>160</v>
       </c>
       <c r="K7">
-        <v>1200000</v>
-      </c>
-      <c r="L7" t="str">
-        <v/>
+        <v>850000</v>
+      </c>
+      <c r="L7">
+        <v>38</v>
       </c>
       <c r="M7">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N7" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Y</v>
+      </c>
+      <c r="P7" t="str">
         <v>N</v>
-      </c>
-      <c r="O7" t="str">
-        <v>N</v>
-      </c>
-      <c r="P7" t="str">
-        <v>Y</v>
       </c>
       <c r="Q7" t="str">
         <v>Y</v>
@@ -1395,7 +1395,7 @@
         <v>Parent</v>
       </c>
       <c r="AP7" t="str">
-        <v>2526QAQD-002</v>
+        <v>2526QAQD-001</v>
       </c>
       <c r="AQ7" t="str">
         <v/>
@@ -1404,51 +1404,51 @@
         <v/>
       </c>
       <c r="AS7" t="str">
-        <v>2526QAQD-002</v>
+        <v>2526QAQD-001</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>2425QAQD-001</v>
+        <v>2526QAQD-002</v>
       </c>
       <c r="B8" t="str">
-        <v>Customer Complaint Analytics</v>
+        <v>SAP HR Module Integration</v>
       </c>
       <c r="C8" t="str">
-        <v>Customer Experience</v>
+        <v>Operational Excellence</v>
       </c>
       <c r="D8" t="str">
-        <v>Customer Service</v>
+        <v>HR</v>
       </c>
       <c r="E8" t="str">
-        <v>IL4</v>
+        <v>IL2</v>
       </c>
       <c r="F8" t="str">
-        <v>Analytics</v>
+        <v>Integration</v>
       </c>
       <c r="G8" t="str">
-        <v>2024-25</v>
+        <v>2025-26</v>
       </c>
       <c r="H8" t="str">
-        <v>2025-06-30</v>
+        <v>2026-03-31</v>
       </c>
       <c r="I8" t="str">
-        <v>2025-07-15</v>
+        <v/>
       </c>
       <c r="J8">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="K8">
-        <v>340000</v>
-      </c>
-      <c r="L8">
-        <v>55</v>
+        <v>1200000</v>
+      </c>
+      <c r="L8" t="str">
+        <v/>
       </c>
       <c r="M8">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="N8" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="O8" t="str">
         <v>N</v>
@@ -1532,7 +1532,7 @@
         <v>Parent</v>
       </c>
       <c r="AP8" t="str">
-        <v>2425QAQD-001</v>
+        <v>2526QAQD-002</v>
       </c>
       <c r="AQ8" t="str">
         <v/>
@@ -1541,60 +1541,60 @@
         <v/>
       </c>
       <c r="AS8" t="str">
-        <v>2425QAQD-001</v>
+        <v>2526QAQD-002</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>2425QAQD-002</v>
+        <v>2425QAQD-001</v>
       </c>
       <c r="B9" t="str">
-        <v>Supply Chain Visibility Dashboard</v>
+        <v>Customer Complaint Analytics</v>
       </c>
       <c r="C9" t="str">
-        <v>Data &amp; Analytics</v>
+        <v>Customer Experience</v>
       </c>
       <c r="D9" t="str">
-        <v>Supply Chain</v>
+        <v>Customer Service</v>
       </c>
       <c r="E9" t="str">
-        <v>Live</v>
+        <v>IL4</v>
       </c>
       <c r="F9" t="str">
-        <v>Reporting</v>
+        <v>Analytics</v>
       </c>
       <c r="G9" t="str">
         <v>2024-25</v>
       </c>
       <c r="H9" t="str">
-        <v>2025-03-31</v>
+        <v>2025-06-30</v>
       </c>
       <c r="I9" t="str">
-        <v>2025-03-28</v>
+        <v>2025-07-15</v>
       </c>
       <c r="J9">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="K9">
-        <v>675000</v>
+        <v>340000</v>
       </c>
       <c r="L9">
-        <v>72</v>
+        <v>55</v>
       </c>
       <c r="M9">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="N9" t="str">
         <v>Y</v>
       </c>
       <c r="O9" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="P9" t="str">
         <v>Y</v>
       </c>
       <c r="Q9" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="R9" t="str">
         <v/>
@@ -1669,7 +1669,7 @@
         <v>Parent</v>
       </c>
       <c r="AP9" t="str">
-        <v>2425QAQD-002</v>
+        <v>2425QAQD-001</v>
       </c>
       <c r="AQ9" t="str">
         <v/>
@@ -1678,57 +1678,57 @@
         <v/>
       </c>
       <c r="AS9" t="str">
-        <v>2425QAQD-002</v>
+        <v>2425QAQD-001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>2425QAQD-003</v>
+        <v>2425QAQD-002</v>
       </c>
       <c r="B10" t="str">
-        <v>AI Dashboard</v>
+        <v>Supply Chain Visibility Dashboard</v>
       </c>
       <c r="C10" t="str">
-        <v>Regulatory Compliance</v>
+        <v>Data &amp; Analytics</v>
       </c>
       <c r="D10" t="str">
-        <v>Marketing</v>
+        <v>Supply Chain</v>
       </c>
       <c r="E10" t="str">
-        <v>IL5</v>
+        <v>Live</v>
       </c>
       <c r="F10" t="str">
-        <v>Innovation</v>
+        <v>Reporting</v>
       </c>
       <c r="G10" t="str">
         <v>2024-25</v>
       </c>
       <c r="H10" t="str">
-        <v>2024-10-12</v>
+        <v>2025-03-31</v>
       </c>
       <c r="I10" t="str">
-        <v>2024-11-10</v>
+        <v>2025-03-28</v>
       </c>
       <c r="J10">
-        <v>14</v>
+        <v>200</v>
       </c>
       <c r="K10">
-        <v>15999</v>
+        <v>675000</v>
       </c>
       <c r="L10">
-        <v>12</v>
+        <v>72</v>
       </c>
       <c r="M10">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="N10" t="str">
         <v>Y</v>
       </c>
       <c r="O10" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="P10" t="str">
-        <v>N</v>
+        <v>Y</v>
       </c>
       <c r="Q10" t="str">
         <v>N</v>
@@ -1806,7 +1806,7 @@
         <v>Parent</v>
       </c>
       <c r="AP10" t="str">
-        <v>2425QAQD-003</v>
+        <v>2425QAQD-002</v>
       </c>
       <c r="AQ10" t="str">
         <v/>
@@ -1815,57 +1815,57 @@
         <v/>
       </c>
       <c r="AS10" t="str">
-        <v>2425QAQD-003</v>
+        <v>2425QAQD-002</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>2627QAQD-002</v>
+        <v>2425QAQD-003</v>
       </c>
       <c r="B11" t="str">
-        <v>AI DASH</v>
+        <v>AI Dashboard</v>
       </c>
       <c r="C11" t="str">
-        <v>Customer Experience</v>
+        <v>Regulatory Compliance</v>
       </c>
       <c r="D11" t="str">
-        <v>IT</v>
+        <v>Marketing</v>
       </c>
       <c r="E11" t="str">
-        <v>Live</v>
+        <v>IL5</v>
       </c>
       <c r="F11" t="str">
-        <v>Compliance</v>
+        <v>Innovation</v>
       </c>
       <c r="G11" t="str">
-        <v>2026-27</v>
+        <v>2024-25</v>
       </c>
       <c r="H11" t="str">
-        <v>2026-08-10</v>
+        <v>2024-10-12</v>
       </c>
       <c r="I11" t="str">
-        <v>2026-06-21</v>
+        <v>2024-11-10</v>
       </c>
       <c r="J11">
-        <v>120</v>
+        <v>14</v>
       </c>
       <c r="K11">
-        <v>45000</v>
+        <v>15999</v>
       </c>
       <c r="L11">
-        <v>38</v>
+        <v>12</v>
       </c>
       <c r="M11">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="N11" t="str">
         <v>Y</v>
       </c>
       <c r="O11" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="P11" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="Q11" t="str">
         <v>N</v>
@@ -1943,21 +1943,158 @@
         <v>Parent</v>
       </c>
       <c r="AP11" t="str">
+        <v>2425QAQD-003</v>
+      </c>
+      <c r="AQ11" t="str">
+        <v/>
+      </c>
+      <c r="AR11" t="str">
+        <v/>
+      </c>
+      <c r="AS11" t="str">
+        <v>2425QAQD-003</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
         <v>2627QAQD-002</v>
       </c>
-      <c r="AQ11" t="str">
-        <v/>
-      </c>
-      <c r="AR11" t="str">
-        <v/>
-      </c>
-      <c r="AS11" t="str">
+      <c r="B12" t="str">
+        <v>AI DASH</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Customer Experience</v>
+      </c>
+      <c r="D12" t="str">
+        <v>IT</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Live</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Compliance</v>
+      </c>
+      <c r="G12" t="str">
+        <v>2026-27</v>
+      </c>
+      <c r="H12" t="str">
+        <v>2026-08-10</v>
+      </c>
+      <c r="I12" t="str">
+        <v>2026-06-21</v>
+      </c>
+      <c r="J12">
+        <v>120</v>
+      </c>
+      <c r="K12">
+        <v>45000</v>
+      </c>
+      <c r="L12">
+        <v>38</v>
+      </c>
+      <c r="M12">
+        <v>12</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Y</v>
+      </c>
+      <c r="O12" t="str">
+        <v>Y</v>
+      </c>
+      <c r="P12" t="str">
+        <v>Y</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>N</v>
+      </c>
+      <c r="R12" t="str">
+        <v/>
+      </c>
+      <c r="S12" t="str">
+        <v/>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v/>
+      </c>
+      <c r="V12" t="str">
+        <v/>
+      </c>
+      <c r="W12" t="str">
+        <v/>
+      </c>
+      <c r="X12" t="str">
+        <v/>
+      </c>
+      <c r="Y12" t="str">
+        <v/>
+      </c>
+      <c r="Z12" t="str">
+        <v/>
+      </c>
+      <c r="AA12" t="str">
+        <v/>
+      </c>
+      <c r="AB12" t="str">
+        <v/>
+      </c>
+      <c r="AC12" t="str">
+        <v/>
+      </c>
+      <c r="AD12" t="str">
+        <v/>
+      </c>
+      <c r="AE12" t="str">
+        <v/>
+      </c>
+      <c r="AF12" t="str">
+        <v/>
+      </c>
+      <c r="AG12" t="str">
+        <v/>
+      </c>
+      <c r="AH12" t="str">
+        <v/>
+      </c>
+      <c r="AI12" t="str">
+        <v/>
+      </c>
+      <c r="AJ12" t="str">
+        <v/>
+      </c>
+      <c r="AK12" t="str">
+        <v/>
+      </c>
+      <c r="AL12" t="str">
+        <v/>
+      </c>
+      <c r="AM12" t="str">
+        <v/>
+      </c>
+      <c r="AN12" t="str">
+        <v/>
+      </c>
+      <c r="AO12" t="str">
+        <v>Parent</v>
+      </c>
+      <c r="AP12" t="str">
+        <v>2627QAQD-002</v>
+      </c>
+      <c r="AQ12" t="str">
+        <v/>
+      </c>
+      <c r="AR12" t="str">
+        <v/>
+      </c>
+      <c r="AS12" t="str">
         <v>2627QAQD-002</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AS11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AS12"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat: Add PIC Staleness Tracker page
</commit_message>
<xml_diff>
--- a/PMO_Master.xlsx
+++ b/PMO_Master.xlsx
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:BB2"/>
+  <dimension ref="A1:BB1"/>
   <cols>
     <col min="1" max="1" hidden="true"/>
     <col min="2" max="2" hidden="true"/>
@@ -621,173 +621,9 @@
         <v>Third Party</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Parent</v>
-      </c>
-      <c r="C2" t="str">
-        <v>2425QAQD-001</v>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v/>
-      </c>
-      <c r="F2" t="str">
-        <v>2425QAQD-001</v>
-      </c>
-      <c r="G2" t="str">
-        <v>N</v>
-      </c>
-      <c r="H2" t="str">
-        <v>N</v>
-      </c>
-      <c r="I2" t="str">
-        <v>hello</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Enterprise Level</v>
-      </c>
-      <c r="K2" t="str">
-        <v>IL4</v>
-      </c>
-      <c r="L2" t="str">
-        <v>GenAI</v>
-      </c>
-      <c r="M2" t="str">
-        <v>PQ-MP</v>
-      </c>
-      <c r="N2" t="str">
-        <v/>
-      </c>
-      <c r="O2" t="str">
-        <v>2024-25</v>
-      </c>
-      <c r="P2" t="str">
-        <v/>
-      </c>
-      <c r="Q2" t="str">
-        <v/>
-      </c>
-      <c r="R2">
-        <v>10</v>
-      </c>
-      <c r="S2" t="str">
-        <v/>
-      </c>
-      <c r="T2" t="str">
-        <v/>
-      </c>
-      <c r="U2" t="str">
-        <v/>
-      </c>
-      <c r="V2" t="str">
-        <v/>
-      </c>
-      <c r="W2" t="str">
-        <v/>
-      </c>
-      <c r="X2" t="str">
-        <v/>
-      </c>
-      <c r="Y2" t="str">
-        <v/>
-      </c>
-      <c r="Z2" t="str">
-        <v/>
-      </c>
-      <c r="AA2" t="str">
-        <v/>
-      </c>
-      <c r="AB2" t="str">
-        <v/>
-      </c>
-      <c r="AC2" t="str">
-        <v/>
-      </c>
-      <c r="AD2" t="str">
-        <v/>
-      </c>
-      <c r="AE2" t="str">
-        <v/>
-      </c>
-      <c r="AF2" t="str">
-        <v/>
-      </c>
-      <c r="AG2" t="str">
-        <v/>
-      </c>
-      <c r="AH2" t="str">
-        <v/>
-      </c>
-      <c r="AI2" t="str">
-        <v/>
-      </c>
-      <c r="AJ2" t="str">
-        <v/>
-      </c>
-      <c r="AK2" t="str">
-        <v/>
-      </c>
-      <c r="AL2" t="str">
-        <v/>
-      </c>
-      <c r="AM2" t="str">
-        <v/>
-      </c>
-      <c r="AN2" t="str">
-        <v/>
-      </c>
-      <c r="AO2" t="str">
-        <v/>
-      </c>
-      <c r="AP2" t="str">
-        <v/>
-      </c>
-      <c r="AQ2" t="str">
-        <v/>
-      </c>
-      <c r="AR2" t="str">
-        <v/>
-      </c>
-      <c r="AS2" t="str">
-        <v/>
-      </c>
-      <c r="AT2" t="str">
-        <v/>
-      </c>
-      <c r="AU2" t="str">
-        <v/>
-      </c>
-      <c r="AV2" t="str">
-        <v/>
-      </c>
-      <c r="AW2" t="str">
-        <v/>
-      </c>
-      <c r="AX2" t="str">
-        <v/>
-      </c>
-      <c r="AY2" t="str">
-        <v>Hello (pic)</v>
-      </c>
-      <c r="AZ2" t="str">
-        <v/>
-      </c>
-      <c r="BA2" t="str">
-        <v>N</v>
-      </c>
-      <c r="BB2" t="str">
-        <v>N</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:BB2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:BB1"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>